<commit_message>
docs: expand beat metrics sheet — DM/post/feed/gate outcomes per choice
Added 7 columns to 'Beats — full consequences': Outcome type (DM/Post/Gate),
DM → to whom, DM text, Post (who + caption), Feed reaction (who + caption),
Gate pass/fail (threshold + assists + what each branch fires), runWrite. Now
every choice shows its full output, not just meter deltas.

Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/cricket-beats-metrics.xlsx
+++ b/docs/cricket-beats-metrics.xlsx
@@ -7,11 +7,11 @@
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Beats — metric consequences" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Beats — full consequences" sheetId="1" state="visible" r:id="rId1"/>
     <sheet name="Reference" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Beats — metric consequences'!$A$1:$L$1</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Beats — full consequences'!$A$1:$Q$1</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -20,7 +20,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="7">
+  <fonts count="5">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -31,7 +31,7 @@
     <font>
       <b val="1"/>
       <color rgb="00FFFFFF"/>
-      <sz val="11"/>
+      <sz val="10"/>
     </font>
     <font>
       <color rgb="00B00020"/>
@@ -43,14 +43,6 @@
       <b val="1"/>
       <color rgb="00003087"/>
       <sz val="14"/>
-    </font>
-    <font>
-      <b val="1"/>
-      <color rgb="00003087"/>
-      <sz val="12"/>
-    </font>
-    <font>
-      <b val="1"/>
     </font>
   </fonts>
   <fills count="4">
@@ -97,44 +89,42 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="15">
+  <cellXfs count="13">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment vertical="center"/>
+      <alignment vertical="top"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment vertical="center" wrapText="1"/>
+      <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
+      <alignment horizontal="center" vertical="top"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
+      <alignment horizontal="center" vertical="top"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment vertical="center"/>
+      <alignment vertical="top"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment vertical="center" wrapText="1"/>
+      <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
+      <alignment horizontal="center" vertical="top"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
+      <alignment horizontal="center" vertical="top"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
+      <alignment horizontal="center" vertical="top"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
+      <alignment horizontal="center" vertical="top"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -500,24 +490,29 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L49"/>
+  <dimension ref="A1:Q49"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="9" customWidth="1" min="1" max="1"/>
-    <col width="6" customWidth="1" min="2" max="2"/>
-    <col width="14" customWidth="1" min="3" max="3"/>
-    <col width="22" customWidth="1" min="4" max="4"/>
-    <col width="15" customWidth="1" min="5" max="5"/>
-    <col width="7" customWidth="1" min="6" max="6"/>
-    <col width="46" customWidth="1" min="7" max="7"/>
-    <col width="8" customWidth="1" min="8" max="8"/>
-    <col width="8" customWidth="1" min="9" max="9"/>
+    <col width="8" customWidth="1" min="1" max="1"/>
+    <col width="4" customWidth="1" min="2" max="2"/>
+    <col width="20" customWidth="1" min="3" max="3"/>
+    <col width="12" customWidth="1" min="4" max="4"/>
+    <col width="7" customWidth="1" min="5" max="5"/>
+    <col width="40" customWidth="1" min="6" max="6"/>
+    <col width="7" customWidth="1" min="7" max="7"/>
+    <col width="7" customWidth="1" min="8" max="8"/>
+    <col width="9" customWidth="1" min="9" max="9"/>
     <col width="20" customWidth="1" min="10" max="10"/>
-    <col width="26" customWidth="1" min="11" max="11"/>
-    <col width="30" customWidth="1" min="12" max="12"/>
+    <col width="9" customWidth="1" min="11" max="11"/>
+    <col width="16" customWidth="1" min="12" max="12"/>
+    <col width="44" customWidth="1" min="13" max="13"/>
+    <col width="44" customWidth="1" min="14" max="14"/>
+    <col width="44" customWidth="1" min="15" max="15"/>
+    <col width="44" customWidth="1" min="16" max="16"/>
+    <col width="10" customWidth="1" min="17" max="17"/>
   </cols>
   <sheetData>
-    <row r="1" ht="32" customHeight="1">
+    <row r="1" ht="40" customHeight="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
           <t>Beat</t>
@@ -525,57 +520,82 @@
       </c>
       <c r="B1" s="1" t="inlineStr">
         <is>
-          <t>Week</t>
+          <t>Wk</t>
         </is>
       </c>
       <c r="C1" s="1" t="inlineStr">
         <is>
-          <t>Week name</t>
+          <t>Title</t>
         </is>
       </c>
       <c r="D1" s="1" t="inlineStr">
         <is>
-          <t>Title</t>
+          <t>Path</t>
         </is>
       </c>
       <c r="E1" s="1" t="inlineStr">
         <is>
-          <t>Path</t>
+          <t>Choice</t>
         </is>
       </c>
       <c r="F1" s="1" t="inlineStr">
         <is>
-          <t>Choice</t>
+          <t>Choice text</t>
         </is>
       </c>
       <c r="G1" s="1" t="inlineStr">
         <is>
-          <t>Choice text</t>
+          <t>Form Δ</t>
         </is>
       </c>
       <c r="H1" s="1" t="inlineStr">
         <is>
-          <t>Form Δ</t>
+          <t>Fame Δ</t>
         </is>
       </c>
       <c r="I1" s="1" t="inlineStr">
         <is>
-          <t>Fame Δ</t>
+          <t>Captain Δ</t>
         </is>
       </c>
       <c r="J1" s="1" t="inlineStr">
         <is>
-          <t>Captain (Hardik) trust Δ</t>
+          <t>Other trust Δ</t>
         </is>
       </c>
       <c r="K1" s="1" t="inlineStr">
         <is>
-          <t>Other seniors trust Δ</t>
+          <t>Outcome</t>
         </is>
       </c>
       <c r="L1" s="1" t="inlineStr">
         <is>
-          <t>Gate / outcome</t>
+          <t>DM → to whom</t>
+        </is>
+      </c>
+      <c r="M1" s="1" t="inlineStr">
+        <is>
+          <t>DM (text)</t>
+        </is>
+      </c>
+      <c r="N1" s="1" t="inlineStr">
+        <is>
+          <t>Post (who: caption)</t>
+        </is>
+      </c>
+      <c r="O1" s="1" t="inlineStr">
+        <is>
+          <t>Feed reaction (who: caption)</t>
+        </is>
+      </c>
+      <c r="P1" s="1" t="inlineStr">
+        <is>
+          <t>Gate (pass/fail)</t>
+        </is>
+      </c>
+      <c r="Q1" s="1" t="inlineStr">
+        <is>
+          <t>runWrite</t>
         </is>
       </c>
     </row>
@@ -590,44 +610,61 @@
       </c>
       <c r="C2" s="2" t="inlineStr">
         <is>
-          <t>Arrival</t>
+          <t>Sold. Mumbai.</t>
         </is>
       </c>
       <c r="D2" s="2" t="inlineStr">
         <is>
-          <t>Sold. Mumbai.</t>
+          <t>default</t>
         </is>
       </c>
       <c r="E2" s="2" t="inlineStr">
         <is>
-          <t>default</t>
-        </is>
-      </c>
-      <c r="F2" s="2" t="inlineStr">
-        <is>
           <t>A</t>
         </is>
       </c>
-      <c r="G2" s="3" t="inlineStr">
+      <c r="F2" s="3" t="inlineStr">
         <is>
           <t>Phone band. Family pehle.</t>
         </is>
       </c>
-      <c r="H2" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="I2" s="5" t="n">
+      <c r="G2" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="H2" s="5" t="n">
         <v>-1</v>
       </c>
-      <c r="J2" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="K2" s="3" t="inlineStr">
+      <c r="I2" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="J2" s="3" t="inlineStr">
         <is>
           <t>friend +2</t>
         </is>
       </c>
-      <c r="L2" s="3" t="inlineStr"/>
+      <c r="K2" s="2" t="inlineStr">
+        <is>
+          <t>DM</t>
+        </is>
+      </c>
+      <c r="L2" s="2" t="inlineStr">
+        <is>
+          <t>friend ×3</t>
+        </is>
+      </c>
+      <c r="M2" s="3" t="inlineStr">
+        <is>
+          <t>11 baar call kiya aur tu family ke saath tha. Correct hai bro. Main khush bhi hoon, jealous bhi hoon, thoda emotional bhi 😭 | Mummy ro rahi thi na? V…</t>
+        </is>
+      </c>
+      <c r="N2" s="3" t="inlineStr"/>
+      <c r="O2" s="3" t="inlineStr">
+        <is>
+          <t>coach: Aaj ek ghar mein TV band hua aur khana garam hua. Sahi shuruaat. Wankhede abhi door hai —…</t>
+        </is>
+      </c>
+      <c r="P2" s="3" t="inlineStr"/>
+      <c r="Q2" s="2" t="inlineStr"/>
     </row>
     <row r="3">
       <c r="A3" s="6" t="inlineStr">
@@ -640,44 +677,65 @@
       </c>
       <c r="C3" s="6" t="inlineStr">
         <is>
-          <t>Arrival</t>
+          <t>Sold. Mumbai.</t>
         </is>
       </c>
       <c r="D3" s="6" t="inlineStr">
         <is>
-          <t>Sold. Mumbai.</t>
+          <t>default</t>
         </is>
       </c>
       <c r="E3" s="6" t="inlineStr">
         <is>
-          <t>default</t>
-        </is>
-      </c>
-      <c r="F3" s="6" t="inlineStr">
-        <is>
           <t>B</t>
         </is>
       </c>
-      <c r="G3" s="7" t="inlineStr">
+      <c r="F3" s="7" t="inlineStr">
         <is>
           <t>Jersey story post karo — abhi</t>
         </is>
       </c>
-      <c r="H3" s="8" t="n">
-        <v>0</v>
-      </c>
-      <c r="I3" s="9" t="n">
+      <c r="G3" s="8" t="n">
+        <v>0</v>
+      </c>
+      <c r="H3" s="9" t="n">
         <v>3</v>
       </c>
-      <c r="J3" s="8" t="n">
-        <v>0</v>
-      </c>
-      <c r="K3" s="7" t="inlineStr">
+      <c r="I3" s="8" t="n">
+        <v>0</v>
+      </c>
+      <c r="J3" s="7" t="inlineStr">
         <is>
           <t>coach -2, friend -2</t>
         </is>
       </c>
-      <c r="L3" s="7" t="inlineStr"/>
+      <c r="K3" s="6" t="inlineStr">
+        <is>
+          <t>POST</t>
+        </is>
+      </c>
+      <c r="L3" s="6" t="inlineStr">
+        <is>
+          <t>friend ×3</t>
+        </is>
+      </c>
+      <c r="M3" s="7" t="inlineStr">
+        <is>
+          <t>Bhai??? 11 missed calls ka reply nahi… aur yeh aa gaya? 😑 | Tu instagram pe duniya se baat kar raha hai aur apne bestie se nahi. Noted. 📝 | Chal thee…</t>
+        </is>
+      </c>
+      <c r="N3" s="7" t="inlineStr">
+        <is>
+          <t>YOU: First time MI jersey haath mein aayi toh samajh nahi aaya smile karun ya ro doon. Academy…</t>
+        </is>
+      </c>
+      <c r="O3" s="7" t="inlineStr">
+        <is>
+          <t>friend: Bro SOLD hua aur 4 minute mein caption ready?? Superstar era officially scary hai 😭</t>
+        </is>
+      </c>
+      <c r="P3" s="7" t="inlineStr"/>
+      <c r="Q3" s="6" t="inlineStr"/>
     </row>
     <row r="4">
       <c r="A4" s="2" t="inlineStr">
@@ -690,44 +748,61 @@
       </c>
       <c r="C4" s="2" t="inlineStr">
         <is>
-          <t>Arrival</t>
+          <t>Bumrah Ka Over</t>
         </is>
       </c>
       <c r="D4" s="2" t="inlineStr">
         <is>
-          <t>Bumrah Ka Over</t>
+          <t>default</t>
         </is>
       </c>
       <c r="E4" s="2" t="inlineStr">
         <is>
-          <t>default</t>
-        </is>
-      </c>
-      <c r="F4" s="2" t="inlineStr">
-        <is>
           <t>A</t>
         </is>
       </c>
-      <c r="G4" s="3" t="inlineStr">
+      <c r="F4" s="3" t="inlineStr">
         <is>
           <t>Defend karo — aur poochho kya miss hua</t>
         </is>
       </c>
-      <c r="H4" s="10" t="n">
+      <c r="G4" s="10" t="n">
         <v>3</v>
       </c>
-      <c r="I4" s="5" t="n">
+      <c r="H4" s="5" t="n">
         <v>-1</v>
       </c>
-      <c r="J4" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="K4" s="3" t="inlineStr">
+      <c r="I4" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="J4" s="3" t="inlineStr">
         <is>
           <t>bumrah +4, rohit +1</t>
         </is>
       </c>
-      <c r="L4" s="3" t="inlineStr"/>
+      <c r="K4" s="2" t="inlineStr">
+        <is>
+          <t>DM</t>
+        </is>
+      </c>
+      <c r="L4" s="2" t="inlineStr">
+        <is>
+          <t>bumrah ×3</t>
+        </is>
+      </c>
+      <c r="M4" s="3" t="inlineStr">
+        <is>
+          <t>Good that you asked. Most don't. | Slower one pe tum ball track kar rahe ho. Galat cheez. Release point track karo — wrist ek beat late girti hai, un…</t>
+        </is>
+      </c>
+      <c r="N4" s="3" t="inlineStr"/>
+      <c r="O4" s="3" t="inlineStr">
+        <is>
+          <t>paltanpulse: Nets update: naya kid Boom se 3 baar beat hua — aur phir POOCHHA kya miss hua. Seniors sa…</t>
+        </is>
+      </c>
+      <c r="P4" s="3" t="inlineStr"/>
+      <c r="Q4" s="2" t="inlineStr"/>
     </row>
     <row r="5">
       <c r="A5" s="6" t="inlineStr">
@@ -740,44 +815,57 @@
       </c>
       <c r="C5" s="6" t="inlineStr">
         <is>
-          <t>Arrival</t>
+          <t>Bumrah Ka Over</t>
         </is>
       </c>
       <c r="D5" s="6" t="inlineStr">
         <is>
-          <t>Bumrah Ka Over</t>
+          <t>default</t>
         </is>
       </c>
       <c r="E5" s="6" t="inlineStr">
         <is>
-          <t>default</t>
-        </is>
-      </c>
-      <c r="F5" s="6" t="inlineStr">
-        <is>
           <t>B</t>
         </is>
       </c>
-      <c r="G5" s="7" t="inlineStr">
+      <c r="F5" s="7" t="inlineStr">
         <is>
           <t>Charge karo — statement shot</t>
         </is>
       </c>
-      <c r="H5" s="11" t="n">
+      <c r="G5" s="11" t="n">
         <v>-2</v>
       </c>
-      <c r="I5" s="9" t="n">
-        <v>2</v>
-      </c>
-      <c r="J5" s="8" t="n">
-        <v>0</v>
-      </c>
-      <c r="K5" s="7" t="inlineStr">
+      <c r="H5" s="9" t="n">
+        <v>2</v>
+      </c>
+      <c r="I5" s="8" t="n">
+        <v>0</v>
+      </c>
+      <c r="J5" s="7" t="inlineStr">
         <is>
           <t>bumrah -2, surya +1</t>
         </is>
       </c>
-      <c r="L5" s="7" t="inlineStr"/>
+      <c r="K5" s="6" t="inlineStr">
+        <is>
+          <t>POST</t>
+        </is>
+      </c>
+      <c r="L5" s="6" t="inlineStr"/>
+      <c r="M5" s="7" t="inlineStr"/>
+      <c r="N5" s="7" t="inlineStr">
+        <is>
+          <t>memeovers: 16-year-old walks into MI nets and CHARGES Jasprit Bumrah on ball four. Missed it by a po…</t>
+        </is>
+      </c>
+      <c r="O5" s="7" t="inlineStr">
+        <is>
+          <t>friend: Bro charged BUMRAH on day one. Legend ya clown — kal pata chalega 😭</t>
+        </is>
+      </c>
+      <c r="P5" s="7" t="inlineStr"/>
+      <c r="Q5" s="6" t="inlineStr"/>
     </row>
     <row r="6">
       <c r="A6" s="2" t="inlineStr">
@@ -790,44 +878,61 @@
       </c>
       <c r="C6" s="2" t="inlineStr">
         <is>
-          <t>Arrival</t>
+          <t>Pehli Press Conference</t>
         </is>
       </c>
       <c r="D6" s="2" t="inlineStr">
         <is>
-          <t>Pehli Press Conference</t>
+          <t>default</t>
         </is>
       </c>
       <c r="E6" s="2" t="inlineStr">
         <is>
-          <t>default</t>
-        </is>
-      </c>
-      <c r="F6" s="2" t="inlineStr">
-        <is>
           <t>A</t>
         </is>
       </c>
-      <c r="G6" s="3" t="inlineStr">
+      <c r="F6" s="3" t="inlineStr">
         <is>
           <t>Team-first seedha jawaab</t>
         </is>
+      </c>
+      <c r="G6" s="10" t="n">
+        <v>1</v>
       </c>
       <c r="H6" s="10" t="n">
         <v>1</v>
       </c>
       <c r="I6" s="10" t="n">
-        <v>1</v>
-      </c>
-      <c r="J6" s="10" t="n">
         <v>3</v>
       </c>
-      <c r="K6" s="3" t="inlineStr">
+      <c r="J6" s="3" t="inlineStr">
         <is>
           <t>mahela +2</t>
         </is>
       </c>
-      <c r="L6" s="3" t="inlineStr"/>
+      <c r="K6" s="2" t="inlineStr">
+        <is>
+          <t>DM</t>
+        </is>
+      </c>
+      <c r="L6" s="2" t="inlineStr">
+        <is>
+          <t>hardik ×2</t>
+        </is>
+      </c>
+      <c r="M6" s="3" t="inlineStr">
+        <is>
+          <t>Presser dekha. Good. No headline. | Bat se shor, mic pe seedha — aise hi khelte hain. Role pe baat jaldi hogi. Tayyar rehna.</t>
+        </is>
+      </c>
+      <c r="N6" s="3" t="inlineStr"/>
+      <c r="O6" s="3" t="inlineStr">
+        <is>
+          <t>naman: Press room mein 2 naye naam the aaj. Slot 1 hai. Kaam bolega. 🤝</t>
+        </is>
+      </c>
+      <c r="P6" s="3" t="inlineStr"/>
+      <c r="Q6" s="2" t="inlineStr"/>
     </row>
     <row r="7">
       <c r="A7" s="6" t="inlineStr">
@@ -840,44 +945,57 @@
       </c>
       <c r="C7" s="6" t="inlineStr">
         <is>
-          <t>Arrival</t>
+          <t>Pehli Press Conference</t>
         </is>
       </c>
       <c r="D7" s="6" t="inlineStr">
         <is>
-          <t>Pehli Press Conference</t>
+          <t>default</t>
         </is>
       </c>
       <c r="E7" s="6" t="inlineStr">
         <is>
-          <t>default</t>
-        </is>
-      </c>
-      <c r="F7" s="6" t="inlineStr">
-        <is>
           <t>B</t>
         </is>
       </c>
-      <c r="G7" s="7" t="inlineStr">
+      <c r="F7" s="7" t="inlineStr">
         <is>
           <t>Headline do</t>
         </is>
       </c>
-      <c r="H7" s="8" t="n">
-        <v>0</v>
-      </c>
-      <c r="I7" s="9" t="n">
+      <c r="G7" s="8" t="n">
+        <v>0</v>
+      </c>
+      <c r="H7" s="9" t="n">
         <v>4</v>
       </c>
-      <c r="J7" s="11" t="n">
+      <c r="I7" s="11" t="n">
         <v>-3</v>
       </c>
-      <c r="K7" s="7" t="inlineStr">
+      <c r="J7" s="7" t="inlineStr">
         <is>
           <t>rohit -1, naman -2</t>
         </is>
       </c>
-      <c r="L7" s="7" t="inlineStr"/>
+      <c r="K7" s="6" t="inlineStr">
+        <is>
+          <t>POST</t>
+        </is>
+      </c>
+      <c r="L7" s="6" t="inlineStr"/>
+      <c r="M7" s="7" t="inlineStr"/>
+      <c r="N7" s="7" t="inlineStr">
+        <is>
+          <t>paltanpulse: "MAIN XI KE LIYE AAYA HOON, WAIT KARNE NAHI." — 16 saal ka confidence ya 16 saal ki galti… || naman: Slot 1 hai. Kaam bolega. 🏏</t>
+        </is>
+      </c>
+      <c r="O7" s="7" t="inlineStr">
+        <is>
+          <t>friend: Bro ek presser mein poora WWE promo maar diya 😭 Mummy ne clip dekha toh kya bolegi socha …</t>
+        </is>
+      </c>
+      <c r="P7" s="7" t="inlineStr"/>
+      <c r="Q7" s="6" t="inlineStr"/>
     </row>
     <row r="8">
       <c r="A8" s="2" t="inlineStr">
@@ -890,44 +1008,61 @@
       </c>
       <c r="C8" s="2" t="inlineStr">
         <is>
-          <t>Arrival</t>
+          <t>Hardik Ka Sawaal</t>
         </is>
       </c>
       <c r="D8" s="2" t="inlineStr">
         <is>
-          <t>Hardik Ka Sawaal</t>
+          <t>default</t>
         </is>
       </c>
       <c r="E8" s="2" t="inlineStr">
         <is>
-          <t>default</t>
-        </is>
-      </c>
-      <c r="F8" s="2" t="inlineStr">
-        <is>
           <t>A</t>
         </is>
       </c>
-      <c r="G8" s="3" t="inlineStr">
+      <c r="F8" s="3" t="inlineStr">
         <is>
           <t>Role accept karo — "Jahan bologe, wahan"</t>
         </is>
       </c>
-      <c r="H8" s="10" t="n">
+      <c r="G8" s="10" t="n">
         <v>1</v>
       </c>
-      <c r="I8" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="J8" s="10" t="n">
+      <c r="H8" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="I8" s="10" t="n">
         <v>5</v>
       </c>
-      <c r="K8" s="3" t="inlineStr">
+      <c r="J8" s="3" t="inlineStr">
         <is>
           <t>mahela +2, tilak +1</t>
         </is>
       </c>
-      <c r="L8" s="3" t="inlineStr"/>
+      <c r="K8" s="2" t="inlineStr">
+        <is>
+          <t>DM</t>
+        </is>
+      </c>
+      <c r="L8" s="2" t="inlineStr">
+        <is>
+          <t>hardik ×2</t>
+        </is>
+      </c>
+      <c r="M8" s="3" t="inlineStr">
+        <is>
+          <t>Good answer. Vague nahi tha. | Jab chance aayega, mujhe flexibility chahiye — explanation nahi. Role clear rakh, sar thanda rakh.</t>
+        </is>
+      </c>
+      <c r="N8" s="3" t="inlineStr"/>
+      <c r="O8" s="3" t="inlineStr">
+        <is>
+          <t>mahela: Young players who understand roles travel faster. Wrote that in a notebook in 2006. Still…</t>
+        </is>
+      </c>
+      <c r="P8" s="3" t="inlineStr"/>
+      <c r="Q8" s="2" t="inlineStr"/>
     </row>
     <row r="9">
       <c r="A9" s="6" t="inlineStr">
@@ -940,44 +1075,57 @@
       </c>
       <c r="C9" s="6" t="inlineStr">
         <is>
-          <t>Arrival</t>
+          <t>Hardik Ka Sawaal</t>
         </is>
       </c>
       <c r="D9" s="6" t="inlineStr">
         <is>
-          <t>Hardik Ka Sawaal</t>
+          <t>default</t>
         </is>
       </c>
       <c r="E9" s="6" t="inlineStr">
         <is>
-          <t>default</t>
-        </is>
-      </c>
-      <c r="F9" s="6" t="inlineStr">
-        <is>
           <t>B</t>
         </is>
       </c>
-      <c r="G9" s="7" t="inlineStr">
+      <c r="F9" s="7" t="inlineStr">
         <is>
           <t>Opening maango — apni strength pitch karo</t>
         </is>
       </c>
-      <c r="H9" s="8" t="n">
-        <v>0</v>
-      </c>
-      <c r="I9" s="9" t="n">
-        <v>2</v>
-      </c>
-      <c r="J9" s="11" t="n">
+      <c r="G9" s="8" t="n">
+        <v>0</v>
+      </c>
+      <c r="H9" s="9" t="n">
+        <v>2</v>
+      </c>
+      <c r="I9" s="11" t="n">
         <v>-4</v>
       </c>
-      <c r="K9" s="7" t="inlineStr">
+      <c r="J9" s="7" t="inlineStr">
         <is>
           <t>rohit -1, naman -1</t>
         </is>
       </c>
-      <c r="L9" s="7" t="inlineStr"/>
+      <c r="K9" s="6" t="inlineStr">
+        <is>
+          <t>POST</t>
+        </is>
+      </c>
+      <c r="L9" s="6" t="inlineStr"/>
+      <c r="M9" s="7" t="inlineStr"/>
+      <c r="N9" s="7" t="inlineStr">
+        <is>
+          <t>futurexi: Inside scoop: MI's teenage buy wants the top order — told the leadership his best use is …</t>
+        </is>
+      </c>
+      <c r="O9" s="7" t="inlineStr">
+        <is>
+          <t>friend: Bro tune HARDIK PANDYA se opening maangi. Built different. Terrifyingly different 😭</t>
+        </is>
+      </c>
+      <c r="P9" s="7" t="inlineStr"/>
+      <c r="Q9" s="6" t="inlineStr"/>
     </row>
     <row r="10">
       <c r="A10" s="2" t="inlineStr">
@@ -990,44 +1138,61 @@
       </c>
       <c r="C10" s="2" t="inlineStr">
         <is>
-          <t>Arrival</t>
+          <t>Team Sheet</t>
         </is>
       </c>
       <c r="D10" s="2" t="inlineStr">
         <is>
-          <t>Team Sheet</t>
+          <t>default</t>
         </is>
       </c>
       <c r="E10" s="2" t="inlineStr">
         <is>
-          <t>default</t>
-        </is>
-      </c>
-      <c r="F10" s="2" t="inlineStr">
-        <is>
           <t>A</t>
         </is>
       </c>
-      <c r="G10" s="3" t="inlineStr">
+      <c r="F10" s="3" t="inlineStr">
         <is>
           <t>Khud jaake batao — seedha, aankhon mein</t>
         </is>
       </c>
-      <c r="H10" s="10" t="n">
+      <c r="G10" s="10" t="n">
         <v>1</v>
       </c>
-      <c r="I10" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="J10" s="10" t="n">
+      <c r="H10" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="I10" s="10" t="n">
         <v>1</v>
       </c>
-      <c r="K10" s="3" t="inlineStr">
+      <c r="J10" s="3" t="inlineStr">
         <is>
           <t>naman +3</t>
         </is>
       </c>
-      <c r="L10" s="3" t="inlineStr"/>
+      <c r="K10" s="2" t="inlineStr">
+        <is>
+          <t>DM</t>
+        </is>
+      </c>
+      <c r="L10" s="2" t="inlineStr">
+        <is>
+          <t>naman ×2</t>
+        </is>
+      </c>
+      <c r="M10" s="3" t="inlineStr">
+        <is>
+          <t>Tu khud bataane aaya. Sheet lagne se pehle. | Jealous hoon, obviously. Par yeh yaad rakhunga. Kal raat jitne over bhi ho, drinks main hi laaunga — ma…</t>
+        </is>
+      </c>
+      <c r="N10" s="3" t="inlineStr"/>
+      <c r="O10" s="3" t="inlineStr">
+        <is>
+          <t>tilak: Sheet ka din sabse zyada batata hai — naam se nahi, reaction se. Aaj kuch reactions note …</t>
+        </is>
+      </c>
+      <c r="P10" s="3" t="inlineStr"/>
+      <c r="Q10" s="2" t="inlineStr"/>
     </row>
     <row r="11">
       <c r="A11" s="6" t="inlineStr">
@@ -1040,44 +1205,57 @@
       </c>
       <c r="C11" s="6" t="inlineStr">
         <is>
-          <t>Arrival</t>
+          <t>Team Sheet</t>
         </is>
       </c>
       <c r="D11" s="6" t="inlineStr">
         <is>
-          <t>Team Sheet</t>
+          <t>default</t>
         </is>
       </c>
       <c r="E11" s="6" t="inlineStr">
         <is>
-          <t>default</t>
-        </is>
-      </c>
-      <c r="F11" s="6" t="inlineStr">
-        <is>
           <t>B</t>
         </is>
       </c>
-      <c r="G11" s="7" t="inlineStr">
+      <c r="F11" s="7" t="inlineStr">
         <is>
           <t>"DEBUT LOADING" story post karo</t>
         </is>
       </c>
-      <c r="H11" s="8" t="n">
-        <v>0</v>
-      </c>
-      <c r="I11" s="9" t="n">
+      <c r="G11" s="8" t="n">
+        <v>0</v>
+      </c>
+      <c r="H11" s="9" t="n">
         <v>3</v>
       </c>
-      <c r="J11" s="11" t="n">
+      <c r="I11" s="11" t="n">
         <v>-2</v>
       </c>
-      <c r="K11" s="7" t="inlineStr">
+      <c r="J11" s="7" t="inlineStr">
         <is>
           <t>naman -2</t>
         </is>
       </c>
-      <c r="L11" s="7" t="inlineStr"/>
+      <c r="K11" s="6" t="inlineStr">
+        <is>
+          <t>POST</t>
+        </is>
+      </c>
+      <c r="L11" s="6" t="inlineStr"/>
+      <c r="M11" s="7" t="inlineStr"/>
+      <c r="N11" s="7" t="inlineStr">
+        <is>
+          <t>YOU: DEBUT LOADING. 🔒🏏 Kal raat. Wankhede. Blue jersey, mera number. Sapna ab schedule pe hai.…</t>
+        </is>
+      </c>
+      <c r="O11" s="7" t="inlineStr">
+        <is>
+          <t>friend: Bro sheet ka screenshot mujhe WhatsApp pe bhejna tha, INSTAGRAM PE NAHI 😭 call me RIGHT N…</t>
+        </is>
+      </c>
+      <c r="P11" s="7" t="inlineStr"/>
+      <c r="Q11" s="6" t="inlineStr"/>
     </row>
     <row r="12">
       <c r="A12" s="2" t="inlineStr">
@@ -1090,40 +1268,57 @@
       </c>
       <c r="C12" s="2" t="inlineStr">
         <is>
-          <t>Arrival</t>
+          <t>Team Sheet</t>
         </is>
       </c>
       <c r="D12" s="2" t="inlineStr">
         <is>
-          <t>Team Sheet</t>
+          <t>LIFELINE</t>
         </is>
       </c>
       <c r="E12" s="2" t="inlineStr">
         <is>
-          <t>LIFELINE path</t>
-        </is>
-      </c>
-      <c r="F12" s="2" t="inlineStr">
-        <is>
           <t>A</t>
         </is>
       </c>
-      <c r="G12" s="3" t="inlineStr">
+      <c r="F12" s="3" t="inlineStr">
         <is>
           <t>Private promise — akele mein Hardik se milo</t>
         </is>
       </c>
-      <c r="H12" s="10" t="n">
+      <c r="G12" s="10" t="n">
         <v>1</v>
       </c>
-      <c r="I12" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="J12" s="10" t="n">
+      <c r="H12" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="I12" s="10" t="n">
         <v>3</v>
       </c>
-      <c r="K12" s="3" t="inlineStr"/>
-      <c r="L12" s="3" t="inlineStr"/>
+      <c r="J12" s="3" t="inlineStr"/>
+      <c r="K12" s="2" t="inlineStr">
+        <is>
+          <t>DM</t>
+        </is>
+      </c>
+      <c r="L12" s="2" t="inlineStr">
+        <is>
+          <t>hardik ×2</t>
+        </is>
+      </c>
+      <c r="M12" s="3" t="inlineStr">
+        <is>
+          <t>Aaya tu. Good. | Sun — yeh charity nahi hai. Maine woh dekha hai jo sheet nahi dikhati. Kal woh dikha de. Aur yeh baat humare beech rahegi.</t>
+        </is>
+      </c>
+      <c r="N12" s="3" t="inlineStr"/>
+      <c r="O12" s="3" t="inlineStr">
+        <is>
+          <t>tilak: Sheet ka din sabse zyada batata hai — naam se nahi, reaction se. Aaj kuch reactions note …</t>
+        </is>
+      </c>
+      <c r="P12" s="3" t="inlineStr"/>
+      <c r="Q12" s="2" t="inlineStr"/>
     </row>
     <row r="13">
       <c r="A13" s="6" t="inlineStr">
@@ -1136,40 +1331,53 @@
       </c>
       <c r="C13" s="6" t="inlineStr">
         <is>
-          <t>Arrival</t>
+          <t>Team Sheet</t>
         </is>
       </c>
       <c r="D13" s="6" t="inlineStr">
         <is>
-          <t>Team Sheet</t>
+          <t>LIFELINE</t>
         </is>
       </c>
       <c r="E13" s="6" t="inlineStr">
         <is>
-          <t>LIFELINE path</t>
-        </is>
-      </c>
-      <c r="F13" s="6" t="inlineStr">
-        <is>
           <t>B</t>
         </is>
       </c>
-      <c r="G13" s="7" t="inlineStr">
+      <c r="F13" s="7" t="inlineStr">
         <is>
           <t>Public thank-you post</t>
         </is>
       </c>
-      <c r="H13" s="8" t="n">
-        <v>0</v>
-      </c>
-      <c r="I13" s="9" t="n">
-        <v>2</v>
-      </c>
-      <c r="J13" s="11" t="n">
+      <c r="G13" s="8" t="n">
+        <v>0</v>
+      </c>
+      <c r="H13" s="9" t="n">
+        <v>2</v>
+      </c>
+      <c r="I13" s="11" t="n">
         <v>-1</v>
       </c>
-      <c r="K13" s="7" t="inlineStr"/>
-      <c r="L13" s="7" t="inlineStr"/>
+      <c r="J13" s="7" t="inlineStr"/>
+      <c r="K13" s="6" t="inlineStr">
+        <is>
+          <t>POST</t>
+        </is>
+      </c>
+      <c r="L13" s="6" t="inlineStr"/>
+      <c r="M13" s="7" t="inlineStr"/>
+      <c r="N13" s="7" t="inlineStr">
+        <is>
+          <t>YOU: Jab numbers ne nahi bola, captain ne bola. @hardikpandya93 — kal raat is bharose ke naam.…</t>
+        </is>
+      </c>
+      <c r="O13" s="7" t="inlineStr">
+        <is>
+          <t>friend: Bro sheet ka screenshot mujhe WhatsApp pe bhejna tha, INSTAGRAM PE NAHI 😭 call me RIGHT N…</t>
+        </is>
+      </c>
+      <c r="P13" s="7" t="inlineStr"/>
+      <c r="Q13" s="6" t="inlineStr"/>
     </row>
     <row r="14">
       <c r="A14" s="2" t="inlineStr">
@@ -1182,44 +1390,61 @@
       </c>
       <c r="C14" s="2" t="inlineStr">
         <is>
-          <t>Arrival</t>
+          <t>Team Sheet</t>
         </is>
       </c>
       <c r="D14" s="2" t="inlineStr">
         <is>
-          <t>Team Sheet</t>
+          <t>BENCHED</t>
         </is>
       </c>
       <c r="E14" s="2" t="inlineStr">
         <is>
-          <t>BENCHED path</t>
-        </is>
-      </c>
-      <c r="F14" s="2" t="inlineStr">
-        <is>
           <t>A</t>
         </is>
       </c>
-      <c r="G14" s="3" t="inlineStr">
+      <c r="F14" s="3" t="inlineStr">
         <is>
           <t>Orange bib, full involvement</t>
         </is>
       </c>
-      <c r="H14" s="10" t="n">
-        <v>2</v>
-      </c>
-      <c r="I14" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="J14" s="10" t="n">
+      <c r="G14" s="10" t="n">
+        <v>2</v>
+      </c>
+      <c r="H14" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="I14" s="10" t="n">
         <v>3</v>
       </c>
-      <c r="K14" s="3" t="inlineStr">
+      <c r="J14" s="3" t="inlineStr">
         <is>
           <t>tilak +1</t>
         </is>
       </c>
-      <c r="L14" s="3" t="inlineStr"/>
+      <c r="K14" s="2" t="inlineStr">
+        <is>
+          <t>DM</t>
+        </is>
+      </c>
+      <c r="L14" s="2" t="inlineStr">
+        <is>
+          <t>tilak ×2</t>
+        </is>
+      </c>
+      <c r="M14" s="3" t="inlineStr">
+        <is>
+          <t>Aaj tujhe drills mein dekha. Bib pehen ke bhi switched on. Naman ko throwdowns tak de raha tha. | Ek cheez bata doon — Hardik bench ko sabse zyada ta…</t>
+        </is>
+      </c>
+      <c r="N14" s="3" t="inlineStr"/>
+      <c r="O14" s="3" t="inlineStr">
+        <is>
+          <t>tilak: Sheet ka din sabse zyada batata hai — naam se nahi, reaction se. Aaj kuch reactions note …</t>
+        </is>
+      </c>
+      <c r="P14" s="3" t="inlineStr"/>
+      <c r="Q14" s="2" t="inlineStr"/>
     </row>
     <row r="15">
       <c r="A15" s="6" t="inlineStr">
@@ -1232,40 +1457,53 @@
       </c>
       <c r="C15" s="6" t="inlineStr">
         <is>
-          <t>Arrival</t>
+          <t>Team Sheet</t>
         </is>
       </c>
       <c r="D15" s="6" t="inlineStr">
         <is>
-          <t>Team Sheet</t>
+          <t>BENCHED</t>
         </is>
       </c>
       <c r="E15" s="6" t="inlineStr">
         <is>
-          <t>BENCHED path</t>
-        </is>
-      </c>
-      <c r="F15" s="6" t="inlineStr">
-        <is>
           <t>B</t>
         </is>
       </c>
-      <c r="G15" s="7" t="inlineStr">
+      <c r="F15" s="7" t="inlineStr">
         <is>
           <t>Outrage posts like karo</t>
         </is>
       </c>
-      <c r="H15" s="8" t="n">
-        <v>0</v>
-      </c>
-      <c r="I15" s="9" t="n">
+      <c r="G15" s="8" t="n">
+        <v>0</v>
+      </c>
+      <c r="H15" s="9" t="n">
         <v>3</v>
       </c>
-      <c r="J15" s="11" t="n">
+      <c r="I15" s="11" t="n">
         <v>-4</v>
       </c>
-      <c r="K15" s="7" t="inlineStr"/>
-      <c r="L15" s="7" t="inlineStr"/>
+      <c r="J15" s="7" t="inlineStr"/>
+      <c r="K15" s="6" t="inlineStr">
+        <is>
+          <t>POST</t>
+        </is>
+      </c>
+      <c r="L15" s="6" t="inlineStr"/>
+      <c r="M15" s="7" t="inlineStr"/>
+      <c r="N15" s="7" t="inlineStr">
+        <is>
+          <t>paltanpulse: 🚨 CONFIRMED: the kid himself has LIKED our benching post. He KNOWS he should be playing. …</t>
+        </is>
+      </c>
+      <c r="O15" s="7" t="inlineStr">
+        <is>
+          <t>friend: Bro sheet ka screenshot mujhe WhatsApp pe bhejna tha, INSTAGRAM PE NAHI 😭 call me RIGHT N…</t>
+        </is>
+      </c>
+      <c r="P15" s="7" t="inlineStr"/>
+      <c r="Q15" s="6" t="inlineStr"/>
     </row>
     <row r="16">
       <c r="A16" s="2" t="inlineStr">
@@ -1278,44 +1516,61 @@
       </c>
       <c r="C16" s="2" t="inlineStr">
         <is>
-          <t>The Debut</t>
+          <t>Debut Morning</t>
         </is>
       </c>
       <c r="D16" s="2" t="inlineStr">
         <is>
-          <t>Debut Morning</t>
+          <t>default</t>
         </is>
       </c>
       <c r="E16" s="2" t="inlineStr">
         <is>
-          <t>default</t>
-        </is>
-      </c>
-      <c r="F16" s="2" t="inlineStr">
-        <is>
           <t>A</t>
         </is>
       </c>
-      <c r="G16" s="3" t="inlineStr">
+      <c r="F16" s="3" t="inlineStr">
         <is>
           <t>Routine pakdo — phone off, shadow practice</t>
         </is>
       </c>
-      <c r="H16" s="10" t="n">
-        <v>2</v>
+      <c r="G16" s="10" t="n">
+        <v>2</v>
+      </c>
+      <c r="H16" s="4" t="n">
+        <v>0</v>
       </c>
       <c r="I16" s="4" t="n">
         <v>0</v>
       </c>
-      <c r="J16" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="K16" s="3" t="inlineStr">
+      <c r="J16" s="3" t="inlineStr">
         <is>
           <t>coach +2</t>
         </is>
       </c>
-      <c r="L16" s="3" t="inlineStr"/>
+      <c r="K16" s="2" t="inlineStr">
+        <is>
+          <t>DM</t>
+        </is>
+      </c>
+      <c r="L16" s="2" t="inlineStr">
+        <is>
+          <t>coach ×3</t>
+        </is>
+      </c>
+      <c r="M16" s="3" t="inlineStr">
+        <is>
+          <t>Video mat bhej beta. Mujhe pata hai tune kiya. Aawaz se pata chal jaata hai. | Aaj sirf teen kaam: pehli ball dekh. Doosri ball dekh. Teesri ball dek…</t>
+        </is>
+      </c>
+      <c r="N16" s="3" t="inlineStr"/>
+      <c r="O16" s="3" t="inlineStr">
+        <is>
+          <t>coach: Matchday pe sabse loud cheez tumhara routine honi chahiye. Baaki sab volume hai.</t>
+        </is>
+      </c>
+      <c r="P16" s="3" t="inlineStr"/>
+      <c r="Q16" s="2" t="inlineStr"/>
     </row>
     <row r="17">
       <c r="A17" s="6" t="inlineStr">
@@ -1328,40 +1583,53 @@
       </c>
       <c r="C17" s="6" t="inlineStr">
         <is>
-          <t>The Debut</t>
+          <t>Debut Morning</t>
         </is>
       </c>
       <c r="D17" s="6" t="inlineStr">
         <is>
-          <t>Debut Morning</t>
+          <t>default</t>
         </is>
       </c>
       <c r="E17" s="6" t="inlineStr">
         <is>
-          <t>default</t>
-        </is>
-      </c>
-      <c r="F17" s="6" t="inlineStr">
-        <is>
           <t>B</t>
         </is>
       </c>
-      <c r="G17" s="7" t="inlineStr">
+      <c r="F17" s="7" t="inlineStr">
         <is>
           <t>Timeline kholo — hype absorb karo</t>
         </is>
       </c>
-      <c r="H17" s="11" t="n">
+      <c r="G17" s="11" t="n">
         <v>-2</v>
       </c>
-      <c r="I17" s="9" t="n">
-        <v>2</v>
-      </c>
-      <c r="J17" s="8" t="n">
-        <v>0</v>
-      </c>
-      <c r="K17" s="7" t="inlineStr"/>
-      <c r="L17" s="7" t="inlineStr"/>
+      <c r="H17" s="9" t="n">
+        <v>2</v>
+      </c>
+      <c r="I17" s="8" t="n">
+        <v>0</v>
+      </c>
+      <c r="J17" s="7" t="inlineStr"/>
+      <c r="K17" s="6" t="inlineStr">
+        <is>
+          <t>POST</t>
+        </is>
+      </c>
+      <c r="L17" s="6" t="inlineStr"/>
+      <c r="M17" s="7" t="inlineStr"/>
+      <c r="N17" s="7" t="inlineStr">
+        <is>
+          <t>paltanpulse: DEBUT DAY 🚨 {name} tonight at Wankhede. 16 saal. Auction se team sheet tak — 3 hafte. Pal…</t>
+        </is>
+      </c>
+      <c r="O17" s="7" t="inlineStr">
+        <is>
+          <t>friend: Bro trending hai aur mujhe chemistry ka test dena hai. Duniya unfair hai 😭 #DebutDay</t>
+        </is>
+      </c>
+      <c r="P17" s="7" t="inlineStr"/>
+      <c r="Q17" s="6" t="inlineStr"/>
     </row>
     <row r="18">
       <c r="A18" s="2" t="inlineStr">
@@ -1374,44 +1642,61 @@
       </c>
       <c r="C18" s="2" t="inlineStr">
         <is>
-          <t>The Debut</t>
+          <t>Debut Morning</t>
         </is>
       </c>
       <c r="D18" s="2" t="inlineStr">
         <is>
-          <t>Debut Morning</t>
+          <t>BENCHED</t>
         </is>
       </c>
       <c r="E18" s="2" t="inlineStr">
         <is>
-          <t>BENCHED path</t>
-        </is>
-      </c>
-      <c r="F18" s="2" t="inlineStr">
-        <is>
           <t>A</t>
         </is>
       </c>
-      <c r="G18" s="3" t="inlineStr">
+      <c r="F18" s="3" t="inlineStr">
         <is>
           <t>Naman ke liye throw-downs do</t>
         </is>
       </c>
-      <c r="H18" s="10" t="n">
+      <c r="G18" s="10" t="n">
         <v>1</v>
       </c>
-      <c r="I18" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="J18" s="10" t="n">
-        <v>2</v>
-      </c>
-      <c r="K18" s="3" t="inlineStr">
+      <c r="H18" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="I18" s="10" t="n">
+        <v>2</v>
+      </c>
+      <c r="J18" s="3" t="inlineStr">
         <is>
           <t>naman +4, tilak +1</t>
         </is>
       </c>
-      <c r="L18" s="3" t="inlineStr"/>
+      <c r="K18" s="2" t="inlineStr">
+        <is>
+          <t>DM</t>
+        </is>
+      </c>
+      <c r="L18" s="2" t="inlineStr">
+        <is>
+          <t>naman ×3</t>
+        </is>
+      </c>
+      <c r="M18" s="3" t="inlineStr">
+        <is>
+          <t>Bhai. Tune chalis minute throw-downs diye. Mere debut ke liye. Apne debut ki jagah. | Yeh main kabhi nahi bhoolunga. Kabhi bhi. | Aaj raat jo bhi ho …</t>
+        </is>
+      </c>
+      <c r="N18" s="3" t="inlineStr"/>
+      <c r="O18" s="3" t="inlineStr">
+        <is>
+          <t>coach: Matchday pe sabse loud cheez tumhara routine honi chahiye. Baaki sab volume hai.</t>
+        </is>
+      </c>
+      <c r="P18" s="3" t="inlineStr"/>
+      <c r="Q18" s="2" t="inlineStr"/>
     </row>
     <row r="19">
       <c r="A19" s="6" t="inlineStr">
@@ -1424,44 +1709,57 @@
       </c>
       <c r="C19" s="6" t="inlineStr">
         <is>
-          <t>The Debut</t>
+          <t>Debut Morning</t>
         </is>
       </c>
       <c r="D19" s="6" t="inlineStr">
         <is>
-          <t>Debut Morning</t>
+          <t>BENCHED</t>
         </is>
       </c>
       <c r="E19" s="6" t="inlineStr">
         <is>
-          <t>BENCHED path</t>
-        </is>
-      </c>
-      <c r="F19" s="6" t="inlineStr">
-        <is>
           <t>B</t>
         </is>
       </c>
-      <c r="G19" s="7" t="inlineStr">
+      <c r="F19" s="7" t="inlineStr">
         <is>
           <t>Apna edit post karo — mid-match</t>
         </is>
       </c>
-      <c r="H19" s="8" t="n">
-        <v>0</v>
-      </c>
-      <c r="I19" s="9" t="n">
+      <c r="G19" s="8" t="n">
+        <v>0</v>
+      </c>
+      <c r="H19" s="9" t="n">
         <v>3</v>
       </c>
-      <c r="J19" s="11" t="n">
+      <c r="I19" s="11" t="n">
         <v>-3</v>
       </c>
-      <c r="K19" s="7" t="inlineStr">
+      <c r="J19" s="7" t="inlineStr">
         <is>
           <t>naman -2</t>
         </is>
       </c>
-      <c r="L19" s="7" t="inlineStr"/>
+      <c r="K19" s="6" t="inlineStr">
+        <is>
+          <t>POST</t>
+        </is>
+      </c>
+      <c r="L19" s="6" t="inlineStr"/>
+      <c r="M19" s="7" t="inlineStr"/>
+      <c r="N19" s="7" t="inlineStr">
+        <is>
+          <t>YOU: Sheet pe naam nahi hai. Story mein hai. Yeh chapter bhi likha jayega. 🔒💙 #Patience</t>
+        </is>
+      </c>
+      <c r="O19" s="7" t="inlineStr">
+        <is>
+          <t>friend: Bro trending hai aur mujhe chemistry ka test dena hai. Duniya unfair hai 😭 #DebutDay</t>
+        </is>
+      </c>
+      <c r="P19" s="7" t="inlineStr"/>
+      <c r="Q19" s="6" t="inlineStr"/>
     </row>
     <row r="20">
       <c r="A20" s="2" t="inlineStr">
@@ -1474,46 +1772,59 @@
       </c>
       <c r="C20" s="2" t="inlineStr">
         <is>
-          <t>The Debut</t>
+          <t>Pehli Gend</t>
         </is>
       </c>
       <c r="D20" s="2" t="inlineStr">
         <is>
-          <t>Pehli Gend</t>
+          <t>default</t>
         </is>
       </c>
       <c r="E20" s="2" t="inlineStr">
         <is>
-          <t>default</t>
-        </is>
-      </c>
-      <c r="F20" s="2" t="inlineStr">
-        <is>
           <t>A</t>
         </is>
       </c>
-      <c r="G20" s="3" t="inlineStr">
+      <c r="F20" s="3" t="inlineStr">
         <is>
           <t>Chase banao — gap, do-lo, phir boundary</t>
         </is>
       </c>
+      <c r="G20" s="10" t="n">
+        <v>3</v>
+      </c>
       <c r="H20" s="10" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="I20" s="10" t="n">
-        <v>1</v>
-      </c>
-      <c r="J20" s="10" t="n">
         <v>4</v>
       </c>
-      <c r="K20" s="3" t="inlineStr">
+      <c r="J20" s="3" t="inlineStr">
         <is>
           <t>rohit +2</t>
         </is>
       </c>
-      <c r="L20" s="3" t="inlineStr">
-        <is>
-          <t>GATE form≥44; assists: bumrah≥34→-4</t>
+      <c r="K20" s="2" t="inlineStr">
+        <is>
+          <t>GATE</t>
+        </is>
+      </c>
+      <c r="L20" s="2" t="inlineStr"/>
+      <c r="M20" s="3" t="inlineStr"/>
+      <c r="N20" s="3" t="inlineStr"/>
+      <c r="O20" s="3" t="inlineStr">
+        <is>
+          <t>rohit: Pehli raat sab kuch nahi hoti. Par pehli raat pe jo dikhta hai, woh jhooth nahi hota.</t>
+        </is>
+      </c>
+      <c r="P20" s="3" t="inlineStr">
+        <is>
+          <t>GATE form≥44 | assists: bumrah≥34→-4 | PASS: '47 OFF 29' feed post | FAIL: '9 OFF 11' DM rohit ×2</t>
+        </is>
+      </c>
+      <c r="Q20" s="2" t="inlineStr">
+        <is>
+          <t>debut</t>
         </is>
       </c>
     </row>
@@ -1528,46 +1839,59 @@
       </c>
       <c r="C21" s="6" t="inlineStr">
         <is>
-          <t>The Debut</t>
+          <t>Pehli Gend</t>
         </is>
       </c>
       <c r="D21" s="6" t="inlineStr">
         <is>
-          <t>Pehli Gend</t>
+          <t>default</t>
         </is>
       </c>
       <c r="E21" s="6" t="inlineStr">
         <is>
-          <t>default</t>
-        </is>
-      </c>
-      <c r="F21" s="6" t="inlineStr">
-        <is>
           <t>B</t>
         </is>
       </c>
-      <c r="G21" s="7" t="inlineStr">
+      <c r="F21" s="7" t="inlineStr">
         <is>
           <t>Counter-attack — pehle over se announce karo</t>
         </is>
       </c>
+      <c r="G21" s="9" t="n">
+        <v>1</v>
+      </c>
       <c r="H21" s="9" t="n">
+        <v>3</v>
+      </c>
+      <c r="I21" s="9" t="n">
         <v>1</v>
       </c>
-      <c r="I21" s="9" t="n">
-        <v>3</v>
-      </c>
-      <c r="J21" s="9" t="n">
-        <v>1</v>
-      </c>
-      <c r="K21" s="7" t="inlineStr">
+      <c r="J21" s="7" t="inlineStr">
         <is>
           <t>surya +2</t>
         </is>
       </c>
-      <c r="L21" s="7" t="inlineStr">
-        <is>
-          <t>GATE form≥44; assists: bumrah≥34→-4</t>
+      <c r="K21" s="6" t="inlineStr">
+        <is>
+          <t>GATE</t>
+        </is>
+      </c>
+      <c r="L21" s="6" t="inlineStr"/>
+      <c r="M21" s="7" t="inlineStr"/>
+      <c r="N21" s="7" t="inlineStr"/>
+      <c r="O21" s="7" t="inlineStr">
+        <is>
+          <t>friend: Bro ka pehla MI matchday tha aaj. Main abhi tak normal nahi hua. Shayad kabhi nahi hounga.</t>
+        </is>
+      </c>
+      <c r="P21" s="7" t="inlineStr">
+        <is>
+          <t>GATE form≥44 | assists: bumrah≥34→-4 | PASS: '38 OFF 16' feed post | FAIL: '2 OFF 3' DM surya ×2</t>
+        </is>
+      </c>
+      <c r="Q21" s="6" t="inlineStr">
+        <is>
+          <t>debut</t>
         </is>
       </c>
     </row>
@@ -1582,46 +1906,59 @@
       </c>
       <c r="C22" s="2" t="inlineStr">
         <is>
-          <t>The Debut</t>
+          <t>Pehli Gend</t>
         </is>
       </c>
       <c r="D22" s="2" t="inlineStr">
         <is>
-          <t>Pehli Gend</t>
+          <t>BENCHED</t>
         </is>
       </c>
       <c r="E22" s="2" t="inlineStr">
         <is>
-          <t>BENCHED path</t>
-        </is>
-      </c>
-      <c r="F22" s="2" t="inlineStr">
-        <is>
           <t>A</t>
         </is>
       </c>
-      <c r="G22" s="3" t="inlineStr">
+      <c r="F22" s="3" t="inlineStr">
         <is>
           <t>Pad up karo — switched on raho</t>
         </is>
       </c>
-      <c r="H22" s="10" t="n">
-        <v>2</v>
-      </c>
-      <c r="I22" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="J22" s="10" t="n">
-        <v>2</v>
-      </c>
-      <c r="K22" s="3" t="inlineStr">
+      <c r="G22" s="10" t="n">
+        <v>2</v>
+      </c>
+      <c r="H22" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="I22" s="10" t="n">
+        <v>2</v>
+      </c>
+      <c r="J22" s="3" t="inlineStr">
         <is>
           <t>tilak +1</t>
         </is>
       </c>
-      <c r="L22" s="3" t="inlineStr">
-        <is>
-          <t>GATE charTrust≥46</t>
+      <c r="K22" s="2" t="inlineStr">
+        <is>
+          <t>GATE</t>
+        </is>
+      </c>
+      <c r="L22" s="2" t="inlineStr"/>
+      <c r="M22" s="3" t="inlineStr"/>
+      <c r="N22" s="3" t="inlineStr"/>
+      <c r="O22" s="3" t="inlineStr">
+        <is>
+          <t>rohit: Pehli raat sab kuch nahi hoti. Par pehli raat pe jo dikhta hai, woh jhooth nahi hota.</t>
+        </is>
+      </c>
+      <c r="P22" s="3" t="inlineStr">
+        <is>
+          <t>GATE charTrust≥46 | PASS: 'IMPACT SUB — 14* (8)' feed post | FAIL: 'CALL NAHI AAYA' DM tilak ×3</t>
+        </is>
+      </c>
+      <c r="Q22" s="2" t="inlineStr">
+        <is>
+          <t>debut</t>
         </is>
       </c>
     </row>
@@ -1636,42 +1973,55 @@
       </c>
       <c r="C23" s="6" t="inlineStr">
         <is>
-          <t>The Debut</t>
+          <t>Pehli Gend</t>
         </is>
       </c>
       <c r="D23" s="6" t="inlineStr">
         <is>
-          <t>Pehli Gend</t>
+          <t>BENCHED</t>
         </is>
       </c>
       <c r="E23" s="6" t="inlineStr">
         <is>
-          <t>BENCHED path</t>
-        </is>
-      </c>
-      <c r="F23" s="6" t="inlineStr">
-        <is>
           <t>B</t>
         </is>
       </c>
-      <c r="G23" s="7" t="inlineStr">
+      <c r="F23" s="7" t="inlineStr">
         <is>
           <t>Phone nikaalo — dugout content banao</t>
         </is>
       </c>
-      <c r="H23" s="8" t="n">
-        <v>0</v>
-      </c>
-      <c r="I23" s="9" t="n">
-        <v>2</v>
-      </c>
-      <c r="J23" s="11" t="n">
+      <c r="G23" s="8" t="n">
+        <v>0</v>
+      </c>
+      <c r="H23" s="9" t="n">
+        <v>2</v>
+      </c>
+      <c r="I23" s="11" t="n">
         <v>-3</v>
       </c>
-      <c r="K23" s="7" t="inlineStr"/>
-      <c r="L23" s="7" t="inlineStr">
-        <is>
-          <t>GATE charTrust≥46</t>
+      <c r="J23" s="7" t="inlineStr"/>
+      <c r="K23" s="6" t="inlineStr">
+        <is>
+          <t>GATE</t>
+        </is>
+      </c>
+      <c r="L23" s="6" t="inlineStr"/>
+      <c r="M23" s="7" t="inlineStr"/>
+      <c r="N23" s="7" t="inlineStr"/>
+      <c r="O23" s="7" t="inlineStr">
+        <is>
+          <t>friend: Bro ka pehla MI matchday tha aaj. Main abhi tak normal nahi hua. Shayad kabhi nahi hounga.</t>
+        </is>
+      </c>
+      <c r="P23" s="7" t="inlineStr">
+        <is>
+          <t>GATE charTrust≥46 | PASS: 'BULAYA — PHONE SAMET …' feed post | FAIL: 'CAMERA MEIN SAB AAYA' DM tilak ×2</t>
+        </is>
+      </c>
+      <c r="Q23" s="6" t="inlineStr">
+        <is>
+          <t>debut</t>
         </is>
       </c>
     </row>
@@ -1686,40 +2036,53 @@
       </c>
       <c r="C24" s="2" t="inlineStr">
         <is>
-          <t>The Debut</t>
+          <t>Toofan</t>
         </is>
       </c>
       <c r="D24" s="2" t="inlineStr">
         <is>
-          <t>Toofan</t>
+          <t>default</t>
         </is>
       </c>
       <c r="E24" s="2" t="inlineStr">
         <is>
-          <t>default</t>
-        </is>
-      </c>
-      <c r="F24" s="2" t="inlineStr">
-        <is>
           <t>A</t>
         </is>
       </c>
-      <c r="G24" s="3" t="inlineStr">
+      <c r="F24" s="3" t="inlineStr">
         <is>
           <t>Ride karo — reel, interviews, sab</t>
         </is>
       </c>
-      <c r="H24" s="5" t="n">
+      <c r="G24" s="5" t="n">
         <v>-1</v>
       </c>
-      <c r="I24" s="10" t="n">
+      <c r="H24" s="10" t="n">
         <v>4</v>
       </c>
-      <c r="J24" s="5" t="n">
+      <c r="I24" s="5" t="n">
         <v>-2</v>
       </c>
-      <c r="K24" s="3" t="inlineStr"/>
-      <c r="L24" s="3" t="inlineStr"/>
+      <c r="J24" s="3" t="inlineStr"/>
+      <c r="K24" s="2" t="inlineStr">
+        <is>
+          <t>POST</t>
+        </is>
+      </c>
+      <c r="L24" s="2" t="inlineStr"/>
+      <c r="M24" s="3" t="inlineStr"/>
+      <c r="N24" s="3" t="inlineStr">
+        <is>
+          <t>YOU: Kal raat: Wankhede. Aaj: pura din replay. Sapna tha, ab schedule hai. Yeh toh shuruaat ha…</t>
+        </is>
+      </c>
+      <c r="O24" s="3" t="inlineStr">
+        <is>
+          <t>friend: Timeline ka mood kuch bhi ho — mera banda mera banda hai. 💙</t>
+        </is>
+      </c>
+      <c r="P24" s="3" t="inlineStr"/>
+      <c r="Q24" s="2" t="inlineStr"/>
     </row>
     <row r="25">
       <c r="A25" s="6" t="inlineStr">
@@ -1732,44 +2095,61 @@
       </c>
       <c r="C25" s="6" t="inlineStr">
         <is>
-          <t>The Debut</t>
+          <t>Toofan</t>
         </is>
       </c>
       <c r="D25" s="6" t="inlineStr">
         <is>
-          <t>Toofan</t>
+          <t>default</t>
         </is>
       </c>
       <c r="E25" s="6" t="inlineStr">
         <is>
-          <t>default</t>
-        </is>
-      </c>
-      <c r="F25" s="6" t="inlineStr">
-        <is>
           <t>B</t>
         </is>
       </c>
-      <c r="G25" s="7" t="inlineStr">
+      <c r="F25" s="7" t="inlineStr">
         <is>
           <t>Mute karo — recovery aur review</t>
         </is>
       </c>
-      <c r="H25" s="9" t="n">
-        <v>2</v>
-      </c>
-      <c r="I25" s="8" t="n">
-        <v>0</v>
-      </c>
-      <c r="J25" s="9" t="n">
+      <c r="G25" s="9" t="n">
+        <v>2</v>
+      </c>
+      <c r="H25" s="8" t="n">
+        <v>0</v>
+      </c>
+      <c r="I25" s="9" t="n">
         <v>3</v>
       </c>
-      <c r="K25" s="7" t="inlineStr">
+      <c r="J25" s="7" t="inlineStr">
         <is>
           <t>coach +2</t>
         </is>
       </c>
-      <c r="L25" s="7" t="inlineStr"/>
+      <c r="K25" s="6" t="inlineStr">
+        <is>
+          <t>DM</t>
+        </is>
+      </c>
+      <c r="L25" s="6" t="inlineStr">
+        <is>
+          <t>hardik ×2</t>
+        </is>
+      </c>
+      <c r="M25" s="7" t="inlineStr">
+        <is>
+          <t>Recovery first. Review 10 baje. | Kal raat achhi thi. Aaj se usko repeat karne ka kaam shuru hota hai. Yehi farak hai player aur clip mein.</t>
+        </is>
+      </c>
+      <c r="N25" s="7" t="inlineStr"/>
+      <c r="O25" s="7" t="inlineStr">
+        <is>
+          <t>coach: Shor ke agle din jo nets pe hota hai, wahi career hota hai. Baaki sab mausam hai.</t>
+        </is>
+      </c>
+      <c r="P25" s="7" t="inlineStr"/>
+      <c r="Q25" s="6" t="inlineStr"/>
     </row>
     <row r="26">
       <c r="A26" s="2" t="inlineStr">
@@ -1782,40 +2162,53 @@
       </c>
       <c r="C26" s="2" t="inlineStr">
         <is>
-          <t>The Debut</t>
+          <t>Toofan</t>
         </is>
       </c>
       <c r="D26" s="2" t="inlineStr">
         <is>
-          <t>Toofan</t>
+          <t>if CR2-S7 fail</t>
         </is>
       </c>
       <c r="E26" s="2" t="inlineStr">
         <is>
-          <t>if CR2-S7 fail</t>
-        </is>
-      </c>
-      <c r="F26" s="2" t="inlineStr">
-        <is>
           <t>A</t>
         </is>
       </c>
-      <c r="G26" s="3" t="inlineStr">
+      <c r="F26" s="3" t="inlineStr">
         <is>
           <t>Clap-back post karo</t>
         </is>
       </c>
-      <c r="H26" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="I26" s="10" t="n">
+      <c r="G26" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="H26" s="10" t="n">
         <v>3</v>
       </c>
-      <c r="J26" s="5" t="n">
+      <c r="I26" s="5" t="n">
         <v>-4</v>
       </c>
-      <c r="K26" s="3" t="inlineStr"/>
-      <c r="L26" s="3" t="inlineStr"/>
+      <c r="J26" s="3" t="inlineStr"/>
+      <c r="K26" s="2" t="inlineStr">
+        <is>
+          <t>POST</t>
+        </is>
+      </c>
+      <c r="L26" s="2" t="inlineStr"/>
+      <c r="M26" s="3" t="inlineStr"/>
+      <c r="N26" s="3" t="inlineStr">
+        <is>
+          <t>YOU: 1 raat mein expert ban gaye sab? Meri jersey bhi pehen lo phir. Season lamba hai. Yaad ra…</t>
+        </is>
+      </c>
+      <c r="O26" s="3" t="inlineStr">
+        <is>
+          <t>friend: Timeline ka mood kuch bhi ho — mera banda mera banda hai. 💙</t>
+        </is>
+      </c>
+      <c r="P26" s="3" t="inlineStr"/>
+      <c r="Q26" s="2" t="inlineStr"/>
     </row>
     <row r="27">
       <c r="A27" s="6" t="inlineStr">
@@ -1828,44 +2221,61 @@
       </c>
       <c r="C27" s="6" t="inlineStr">
         <is>
-          <t>The Debut</t>
+          <t>Toofan</t>
         </is>
       </c>
       <c r="D27" s="6" t="inlineStr">
         <is>
-          <t>Toofan</t>
+          <t>if CR2-S7 fail</t>
         </is>
       </c>
       <c r="E27" s="6" t="inlineStr">
         <is>
-          <t>if CR2-S7 fail</t>
-        </is>
-      </c>
-      <c r="F27" s="6" t="inlineStr">
-        <is>
           <t>B</t>
         </is>
       </c>
-      <c r="G27" s="7" t="inlineStr">
+      <c r="F27" s="7" t="inlineStr">
         <is>
           <t>Chup raho — Bumrah se time maango</t>
         </is>
       </c>
-      <c r="H27" s="9" t="n">
+      <c r="G27" s="9" t="n">
         <v>3</v>
       </c>
-      <c r="I27" s="8" t="n">
-        <v>0</v>
-      </c>
-      <c r="J27" s="9" t="n">
-        <v>2</v>
-      </c>
-      <c r="K27" s="7" t="inlineStr">
+      <c r="H27" s="8" t="n">
+        <v>0</v>
+      </c>
+      <c r="I27" s="9" t="n">
+        <v>2</v>
+      </c>
+      <c r="J27" s="7" t="inlineStr">
         <is>
           <t>bumrah +3</t>
         </is>
       </c>
-      <c r="L27" s="7" t="inlineStr"/>
+      <c r="K27" s="6" t="inlineStr">
+        <is>
+          <t>DM</t>
+        </is>
+      </c>
+      <c r="L27" s="6" t="inlineStr">
+        <is>
+          <t>bumrah ×3</t>
+        </is>
+      </c>
+      <c r="M27" s="7" t="inlineStr">
+        <is>
+          <t>Kal subah 7 baje. Nets. Sirf hum do. | Jo timeline keh rahi hai woh data nahi hai. Jo nets mein hoga, woh data hai. | Phone hotel pe chhod ke aana.</t>
+        </is>
+      </c>
+      <c r="N27" s="7" t="inlineStr"/>
+      <c r="O27" s="7" t="inlineStr">
+        <is>
+          <t>coach: Shor ke agle din jo nets pe hota hai, wahi career hota hai. Baaki sab mausam hai.</t>
+        </is>
+      </c>
+      <c r="P27" s="7" t="inlineStr"/>
+      <c r="Q27" s="6" t="inlineStr"/>
     </row>
     <row r="28">
       <c r="A28" s="2" t="inlineStr">
@@ -1878,44 +2288,61 @@
       </c>
       <c r="C28" s="2" t="inlineStr">
         <is>
-          <t>The Debut</t>
+          <t>The Fall</t>
         </is>
       </c>
       <c r="D28" s="2" t="inlineStr">
         <is>
-          <t>The Fall</t>
+          <t>default</t>
         </is>
       </c>
       <c r="E28" s="2" t="inlineStr">
         <is>
-          <t>default</t>
-        </is>
-      </c>
-      <c r="F28" s="2" t="inlineStr">
-        <is>
           <t>A</t>
         </is>
       </c>
-      <c r="G28" s="3" t="inlineStr">
+      <c r="F28" s="3" t="inlineStr">
         <is>
           <t>Own karo — pehle room, phir duniya</t>
         </is>
       </c>
-      <c r="H28" s="10" t="n">
+      <c r="G28" s="10" t="n">
         <v>1</v>
       </c>
-      <c r="I28" s="5" t="n">
+      <c r="H28" s="5" t="n">
         <v>-2</v>
       </c>
-      <c r="J28" s="10" t="n">
+      <c r="I28" s="10" t="n">
         <v>4</v>
       </c>
-      <c r="K28" s="3" t="inlineStr">
+      <c r="J28" s="3" t="inlineStr">
         <is>
           <t>rohit +3</t>
         </is>
       </c>
-      <c r="L28" s="3" t="inlineStr"/>
+      <c r="K28" s="2" t="inlineStr">
+        <is>
+          <t>DM</t>
+        </is>
+      </c>
+      <c r="L28" s="2" t="inlineStr">
+        <is>
+          <t>rohit ×3</t>
+        </is>
+      </c>
+      <c r="M28" s="3" t="inlineStr">
+        <is>
+          <t>Suna maine. Aur yeh bhi suna ki tu khud bolna chahta hai. Achha hai. | Galti sab karte hain. Jawaab kaun deta hai — woh dekha jaata hai. | Kal 9 baje…</t>
+        </is>
+      </c>
+      <c r="N28" s="3" t="inlineStr"/>
+      <c r="O28" s="3" t="inlineStr">
+        <is>
+          <t>hardik: Aaj room ke andar jo hua, woh bahar nahi aayega. Itna bata doon — room handled it. That m…</t>
+        </is>
+      </c>
+      <c r="P28" s="3" t="inlineStr"/>
+      <c r="Q28" s="2" t="inlineStr"/>
     </row>
     <row r="29">
       <c r="A29" s="6" t="inlineStr">
@@ -1928,44 +2355,57 @@
       </c>
       <c r="C29" s="6" t="inlineStr">
         <is>
-          <t>The Debut</t>
+          <t>The Fall</t>
         </is>
       </c>
       <c r="D29" s="6" t="inlineStr">
         <is>
-          <t>The Fall</t>
+          <t>default</t>
         </is>
       </c>
       <c r="E29" s="6" t="inlineStr">
         <is>
-          <t>default</t>
-        </is>
-      </c>
-      <c r="F29" s="6" t="inlineStr">
-        <is>
           <t>B</t>
         </is>
       </c>
-      <c r="G29" s="7" t="inlineStr">
+      <c r="F29" s="7" t="inlineStr">
         <is>
           <t>PR-fix karo — statement post, clips delete</t>
         </is>
       </c>
-      <c r="H29" s="8" t="n">
-        <v>0</v>
-      </c>
-      <c r="I29" s="9" t="n">
-        <v>2</v>
-      </c>
-      <c r="J29" s="11" t="n">
+      <c r="G29" s="8" t="n">
+        <v>0</v>
+      </c>
+      <c r="H29" s="9" t="n">
+        <v>2</v>
+      </c>
+      <c r="I29" s="11" t="n">
         <v>-5</v>
       </c>
-      <c r="K29" s="7" t="inlineStr">
+      <c r="J29" s="7" t="inlineStr">
         <is>
           <t>rohit -2, mahela -2</t>
         </is>
       </c>
-      <c r="L29" s="7" t="inlineStr"/>
+      <c r="K29" s="6" t="inlineStr">
+        <is>
+          <t>POST</t>
+        </is>
+      </c>
+      <c r="L29" s="6" t="inlineStr"/>
+      <c r="M29" s="7" t="inlineStr"/>
+      <c r="N29" s="7" t="inlineStr">
+        <is>
+          <t>YOU: Kal raat se kuch clips circulate ho rahi hain jo bina context ke hain. Meri team is par k…</t>
+        </is>
+      </c>
+      <c r="O29" s="7" t="inlineStr">
+        <is>
+          <t>friend: Bro ka statement dekha. PR wala. Mujhe actual bro se baat karni hai. Actual wale se.</t>
+        </is>
+      </c>
+      <c r="P29" s="7" t="inlineStr"/>
+      <c r="Q29" s="6" t="inlineStr"/>
     </row>
     <row r="30">
       <c r="A30" s="2" t="inlineStr">
@@ -1978,40 +2418,57 @@
       </c>
       <c r="C30" s="2" t="inlineStr">
         <is>
-          <t>The Debut</t>
+          <t>Selection Meeting</t>
         </is>
       </c>
       <c r="D30" s="2" t="inlineStr">
         <is>
-          <t>Selection Meeting</t>
+          <t>default</t>
         </is>
       </c>
       <c r="E30" s="2" t="inlineStr">
         <is>
-          <t>default</t>
-        </is>
-      </c>
-      <c r="F30" s="2" t="inlineStr">
-        <is>
           <t>A</t>
         </is>
       </c>
-      <c r="G30" s="3" t="inlineStr">
+      <c r="F30" s="3" t="inlineStr">
         <is>
           <t>Chup raho — agla match kamao</t>
         </is>
       </c>
-      <c r="H30" s="10" t="n">
-        <v>2</v>
-      </c>
-      <c r="I30" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="J30" s="10" t="n">
-        <v>2</v>
-      </c>
-      <c r="K30" s="3" t="inlineStr"/>
-      <c r="L30" s="3" t="inlineStr"/>
+      <c r="G30" s="10" t="n">
+        <v>2</v>
+      </c>
+      <c r="H30" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="I30" s="10" t="n">
+        <v>2</v>
+      </c>
+      <c r="J30" s="3" t="inlineStr"/>
+      <c r="K30" s="2" t="inlineStr">
+        <is>
+          <t>DM</t>
+        </is>
+      </c>
+      <c r="L30" s="2" t="inlineStr">
+        <is>
+          <t>hardik ×2</t>
+        </is>
+      </c>
+      <c r="M30" s="3" t="inlineStr">
+        <is>
+          <t>Meeting mein jo bola, wahi role hai. No.5. Death tak rukna pade toh rukna. | Aur ek baat. Is hafte tune kuch cheezein sahi ki. Main note karta hoon. …</t>
+        </is>
+      </c>
+      <c r="N30" s="3" t="inlineStr"/>
+      <c r="O30" s="3" t="inlineStr">
+        <is>
+          <t>rohit: Team sheet har hafte ek sawaal poochti hai. Jawaab har hafte dena padta hai.</t>
+        </is>
+      </c>
+      <c r="P30" s="3" t="inlineStr"/>
+      <c r="Q30" s="2" t="inlineStr"/>
     </row>
     <row r="31">
       <c r="A31" s="6" t="inlineStr">
@@ -2024,40 +2481,53 @@
       </c>
       <c r="C31" s="6" t="inlineStr">
         <is>
-          <t>The Debut</t>
+          <t>Selection Meeting</t>
         </is>
       </c>
       <c r="D31" s="6" t="inlineStr">
         <is>
-          <t>Selection Meeting</t>
+          <t>default</t>
         </is>
       </c>
       <c r="E31" s="6" t="inlineStr">
         <is>
-          <t>default</t>
-        </is>
-      </c>
-      <c r="F31" s="6" t="inlineStr">
-        <is>
           <t>B</t>
         </is>
       </c>
-      <c r="G31" s="7" t="inlineStr">
+      <c r="F31" s="7" t="inlineStr">
         <is>
           <t>Vindication post karo</t>
         </is>
       </c>
-      <c r="H31" s="8" t="n">
-        <v>0</v>
-      </c>
-      <c r="I31" s="9" t="n">
+      <c r="G31" s="8" t="n">
+        <v>0</v>
+      </c>
+      <c r="H31" s="9" t="n">
         <v>3</v>
       </c>
-      <c r="J31" s="11" t="n">
+      <c r="I31" s="11" t="n">
         <v>-3</v>
       </c>
-      <c r="K31" s="7" t="inlineStr"/>
-      <c r="L31" s="7" t="inlineStr"/>
+      <c r="J31" s="7" t="inlineStr"/>
+      <c r="K31" s="6" t="inlineStr">
+        <is>
+          <t>POST</t>
+        </is>
+      </c>
+      <c r="L31" s="6" t="inlineStr"/>
+      <c r="M31" s="7" t="inlineStr"/>
+      <c r="N31" s="7" t="inlineStr">
+        <is>
+          <t>YOU: Retained. Jo log 'overhyped' likh rahe the — phir se padh lo. Kaam bolta hai. Hamesha bol…</t>
+        </is>
+      </c>
+      <c r="O31" s="7" t="inlineStr">
+        <is>
+          <t>friend: Bro ka selection saga mera favourite show ban gaya hai. Agla episode Wednesday. 🍿</t>
+        </is>
+      </c>
+      <c r="P31" s="7" t="inlineStr"/>
+      <c r="Q31" s="6" t="inlineStr"/>
     </row>
     <row r="32">
       <c r="A32" s="2" t="inlineStr">
@@ -2070,44 +2540,61 @@
       </c>
       <c r="C32" s="2" t="inlineStr">
         <is>
-          <t>The Debut</t>
+          <t>Selection Meeting</t>
         </is>
       </c>
       <c r="D32" s="2" t="inlineStr">
         <is>
-          <t>Selection Meeting</t>
+          <t>BENCHED</t>
         </is>
       </c>
       <c r="E32" s="2" t="inlineStr">
         <is>
-          <t>BENCHED path</t>
-        </is>
-      </c>
-      <c r="F32" s="2" t="inlineStr">
-        <is>
           <t>A</t>
         </is>
       </c>
-      <c r="G32" s="3" t="inlineStr">
+      <c r="F32" s="3" t="inlineStr">
         <is>
           <t>Naman ke saath kaam karo — number banao</t>
         </is>
       </c>
-      <c r="H32" s="10" t="n">
+      <c r="G32" s="10" t="n">
         <v>3</v>
       </c>
-      <c r="I32" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="J32" s="10" t="n">
-        <v>2</v>
-      </c>
-      <c r="K32" s="3" t="inlineStr">
+      <c r="H32" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="I32" s="10" t="n">
+        <v>2</v>
+      </c>
+      <c r="J32" s="3" t="inlineStr">
         <is>
           <t>naman +3, mahela +2</t>
         </is>
       </c>
-      <c r="L32" s="3" t="inlineStr"/>
+      <c r="K32" s="2" t="inlineStr">
+        <is>
+          <t>DM</t>
+        </is>
+      </c>
+      <c r="L32" s="2" t="inlineStr">
+        <is>
+          <t>mahela ×3</t>
+        </is>
+      </c>
+      <c r="M32" s="3" t="inlineStr">
+        <is>
+          <t>Tumne poocha raasta kya hai. Main seedha bolta hoon. | Form 64 chahiye. Us number pe main selection room mein khud ladta hoon — woh sheet mujhe khud …</t>
+        </is>
+      </c>
+      <c r="N32" s="3" t="inlineStr"/>
+      <c r="O32" s="3" t="inlineStr">
+        <is>
+          <t>rohit: Team sheet har hafte ek sawaal poochti hai. Jawaab har hafte dena padta hai.</t>
+        </is>
+      </c>
+      <c r="P32" s="3" t="inlineStr"/>
+      <c r="Q32" s="2" t="inlineStr"/>
     </row>
     <row r="33">
       <c r="A33" s="6" t="inlineStr">
@@ -2120,44 +2607,57 @@
       </c>
       <c r="C33" s="6" t="inlineStr">
         <is>
-          <t>The Debut</t>
+          <t>Selection Meeting</t>
         </is>
       </c>
       <c r="D33" s="6" t="inlineStr">
         <is>
-          <t>Selection Meeting</t>
+          <t>BENCHED</t>
         </is>
       </c>
       <c r="E33" s="6" t="inlineStr">
         <is>
-          <t>BENCHED path</t>
-        </is>
-      </c>
-      <c r="F33" s="6" t="inlineStr">
-        <is>
           <t>B</t>
         </is>
       </c>
-      <c r="G33" s="7" t="inlineStr">
+      <c r="F33" s="7" t="inlineStr">
         <is>
           <t>Agent ko haan bolo — trade rumor float karo</t>
         </is>
       </c>
-      <c r="H33" s="8" t="n">
-        <v>0</v>
-      </c>
-      <c r="I33" s="9" t="n">
+      <c r="G33" s="8" t="n">
+        <v>0</v>
+      </c>
+      <c r="H33" s="9" t="n">
         <v>4</v>
       </c>
-      <c r="J33" s="11" t="n">
+      <c r="I33" s="11" t="n">
         <v>-6</v>
       </c>
-      <c r="K33" s="7" t="inlineStr">
+      <c r="J33" s="7" t="inlineStr">
         <is>
           <t>mahela -3</t>
         </is>
       </c>
-      <c r="L33" s="7" t="inlineStr"/>
+      <c r="K33" s="6" t="inlineStr">
+        <is>
+          <t>POST</t>
+        </is>
+      </c>
+      <c r="L33" s="6" t="inlineStr"/>
+      <c r="M33" s="7" t="inlineStr"/>
+      <c r="N33" s="7" t="inlineStr">
+        <is>
+          <t>cricketroom_india: EXCLUSIVE: Sources close to the young MI batter say the camp is 'evaluating options' ahea…</t>
+        </is>
+      </c>
+      <c r="O33" s="7" t="inlineStr">
+        <is>
+          <t>friend: Bro ka selection saga mera favourite show ban gaya hai. Agla episode Wednesday. 🍿</t>
+        </is>
+      </c>
+      <c r="P33" s="7" t="inlineStr"/>
+      <c r="Q33" s="6" t="inlineStr"/>
     </row>
     <row r="34">
       <c r="A34" s="2" t="inlineStr">
@@ -2170,40 +2670,57 @@
       </c>
       <c r="C34" s="2" t="inlineStr">
         <is>
-          <t>The Debut</t>
+          <t>Selection Meeting</t>
         </is>
       </c>
       <c r="D34" s="2" t="inlineStr">
         <is>
-          <t>Selection Meeting</t>
+          <t>LIFELINE</t>
         </is>
       </c>
       <c r="E34" s="2" t="inlineStr">
         <is>
-          <t>LIFELINE path</t>
-        </is>
-      </c>
-      <c r="F34" s="2" t="inlineStr">
-        <is>
           <t>A</t>
         </is>
       </c>
-      <c r="G34" s="3" t="inlineStr">
+      <c r="F34" s="3" t="inlineStr">
         <is>
           <t>Private promise — 'is baar numbers'</t>
         </is>
       </c>
-      <c r="H34" s="10" t="n">
+      <c r="G34" s="10" t="n">
         <v>1</v>
       </c>
-      <c r="I34" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="J34" s="10" t="n">
+      <c r="H34" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="I34" s="10" t="n">
         <v>3</v>
       </c>
-      <c r="K34" s="3" t="inlineStr"/>
-      <c r="L34" s="3" t="inlineStr"/>
+      <c r="J34" s="3" t="inlineStr"/>
+      <c r="K34" s="2" t="inlineStr">
+        <is>
+          <t>DM</t>
+        </is>
+      </c>
+      <c r="L34" s="2" t="inlineStr">
+        <is>
+          <t>hardik ×3</t>
+        </is>
+      </c>
+      <c r="M34" s="3" t="inlineStr">
+        <is>
+          <t>Tune message kiya. Good. Zyada log thank-you post karte hain. | Sun. Yeh last explain hai. Ab bat bolega. | Wednesday. No.5. Mujhe innings chahiye, p…</t>
+        </is>
+      </c>
+      <c r="N34" s="3" t="inlineStr"/>
+      <c r="O34" s="3" t="inlineStr">
+        <is>
+          <t>rohit: Team sheet har hafte ek sawaal poochti hai. Jawaab har hafte dena padta hai.</t>
+        </is>
+      </c>
+      <c r="P34" s="3" t="inlineStr"/>
+      <c r="Q34" s="2" t="inlineStr"/>
     </row>
     <row r="35">
       <c r="A35" s="6" t="inlineStr">
@@ -2216,40 +2733,53 @@
       </c>
       <c r="C35" s="6" t="inlineStr">
         <is>
-          <t>The Debut</t>
+          <t>Selection Meeting</t>
         </is>
       </c>
       <c r="D35" s="6" t="inlineStr">
         <is>
-          <t>Selection Meeting</t>
+          <t>LIFELINE</t>
         </is>
       </c>
       <c r="E35" s="6" t="inlineStr">
         <is>
-          <t>LIFELINE path</t>
-        </is>
-      </c>
-      <c r="F35" s="6" t="inlineStr">
-        <is>
           <t>B</t>
         </is>
       </c>
-      <c r="G35" s="7" t="inlineStr">
+      <c r="F35" s="7" t="inlineStr">
         <is>
           <t>Prove-it post karo — publicly</t>
         </is>
       </c>
-      <c r="H35" s="8" t="n">
-        <v>0</v>
-      </c>
-      <c r="I35" s="9" t="n">
-        <v>2</v>
-      </c>
-      <c r="J35" s="11" t="n">
+      <c r="G35" s="8" t="n">
+        <v>0</v>
+      </c>
+      <c r="H35" s="9" t="n">
+        <v>2</v>
+      </c>
+      <c r="I35" s="11" t="n">
         <v>-2</v>
       </c>
-      <c r="K35" s="7" t="inlineStr"/>
-      <c r="L35" s="7" t="inlineStr"/>
+      <c r="J35" s="7" t="inlineStr"/>
+      <c r="K35" s="6" t="inlineStr">
+        <is>
+          <t>POST</t>
+        </is>
+      </c>
+      <c r="L35" s="6" t="inlineStr"/>
+      <c r="M35" s="7" t="inlineStr"/>
+      <c r="N35" s="7" t="inlineStr">
+        <is>
+          <t>YOU: Aaj captain ne mere liye apna naam rakha. Wednesday ko main uska jawaab apne bat se dunga…</t>
+        </is>
+      </c>
+      <c r="O35" s="7" t="inlineStr">
+        <is>
+          <t>friend: Bro ka selection saga mera favourite show ban gaya hai. Agla episode Wednesday. 🍿</t>
+        </is>
+      </c>
+      <c r="P35" s="7" t="inlineStr"/>
+      <c r="Q35" s="6" t="inlineStr"/>
     </row>
     <row r="36">
       <c r="A36" s="2" t="inlineStr">
@@ -2262,44 +2792,61 @@
       </c>
       <c r="C36" s="2" t="inlineStr">
         <is>
-          <t>The Reckoning</t>
+          <t>Akela Hotel Gym</t>
         </is>
       </c>
       <c r="D36" s="2" t="inlineStr">
         <is>
-          <t>Akela Hotel Gym</t>
+          <t>default</t>
         </is>
       </c>
       <c r="E36" s="2" t="inlineStr">
         <is>
-          <t>default</t>
-        </is>
-      </c>
-      <c r="F36" s="2" t="inlineStr">
-        <is>
           <t>A</t>
         </is>
       </c>
-      <c r="G36" s="3" t="inlineStr">
+      <c r="F36" s="3" t="inlineStr">
         <is>
           <t>Coach ke saath wapas basics</t>
         </is>
       </c>
-      <c r="H36" s="10" t="n">
+      <c r="G36" s="10" t="n">
         <v>3</v>
       </c>
+      <c r="H36" s="4" t="n">
+        <v>0</v>
+      </c>
       <c r="I36" s="4" t="n">
         <v>0</v>
       </c>
-      <c r="J36" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="K36" s="3" t="inlineStr">
+      <c r="J36" s="3" t="inlineStr">
         <is>
           <t>coach +3</t>
         </is>
       </c>
-      <c r="L36" s="3" t="inlineStr"/>
+      <c r="K36" s="2" t="inlineStr">
+        <is>
+          <t>DM</t>
+        </is>
+      </c>
+      <c r="L36" s="2" t="inlineStr">
+        <is>
+          <t>coach ×3</t>
+        </is>
+      </c>
+      <c r="M36" s="3" t="inlineStr">
+        <is>
+          <t>Video mila. Wahi dikha jo mujhe lag raha tha — backlift theek hai, base hil gaya hai. Tu ball ke paas jaldi pahunch raha hai. | Kal subah 6 baje vide…</t>
+        </is>
+      </c>
+      <c r="N36" s="3" t="inlineStr"/>
+      <c r="O36" s="3" t="inlineStr">
+        <is>
+          <t>coach: Slump technique se kam, sochne ke tareeke se zyada tootta hai. Mere har student ko ek hi …</t>
+        </is>
+      </c>
+      <c r="P36" s="3" t="inlineStr"/>
+      <c r="Q36" s="2" t="inlineStr"/>
     </row>
     <row r="37">
       <c r="A37" s="6" t="inlineStr">
@@ -2312,40 +2859,53 @@
       </c>
       <c r="C37" s="6" t="inlineStr">
         <is>
-          <t>The Reckoning</t>
+          <t>Akela Hotel Gym</t>
         </is>
       </c>
       <c r="D37" s="6" t="inlineStr">
         <is>
-          <t>Akela Hotel Gym</t>
+          <t>default</t>
         </is>
       </c>
       <c r="E37" s="6" t="inlineStr">
         <is>
-          <t>default</t>
-        </is>
-      </c>
-      <c r="F37" s="6" t="inlineStr">
-        <is>
           <t>B</t>
         </is>
       </c>
-      <c r="G37" s="7" t="inlineStr">
+      <c r="F37" s="7" t="inlineStr">
         <is>
           <t>Lone-wolf grind — aur post karo</t>
         </is>
       </c>
+      <c r="G37" s="9" t="n">
+        <v>1</v>
+      </c>
       <c r="H37" s="9" t="n">
-        <v>1</v>
-      </c>
-      <c r="I37" s="9" t="n">
-        <v>2</v>
-      </c>
-      <c r="J37" s="8" t="n">
-        <v>0</v>
-      </c>
-      <c r="K37" s="7" t="inlineStr"/>
-      <c r="L37" s="7" t="inlineStr"/>
+        <v>2</v>
+      </c>
+      <c r="I37" s="8" t="n">
+        <v>0</v>
+      </c>
+      <c r="J37" s="7" t="inlineStr"/>
+      <c r="K37" s="6" t="inlineStr">
+        <is>
+          <t>POST</t>
+        </is>
+      </c>
+      <c r="L37" s="6" t="inlineStr"/>
+      <c r="M37" s="7" t="inlineStr"/>
+      <c r="N37" s="7" t="inlineStr">
+        <is>
+          <t>YOU: 5 AM. Khaali gym. Koi shortcut nahi, koi excuse nahi. 🔒 #TrustTheProcess</t>
+        </is>
+      </c>
+      <c r="O37" s="7" t="inlineStr">
+        <is>
+          <t>friend: Bhai 5 baje gym story daal raha hai. Main 5 baje so raha hoon. We are not the same. (Prou…</t>
+        </is>
+      </c>
+      <c r="P37" s="7" t="inlineStr"/>
+      <c r="Q37" s="6" t="inlineStr"/>
     </row>
     <row r="38">
       <c r="A38" s="2" t="inlineStr">
@@ -2358,44 +2918,61 @@
       </c>
       <c r="C38" s="2" t="inlineStr">
         <is>
-          <t>The Reckoning</t>
+          <t>Akela Hotel Gym</t>
         </is>
       </c>
       <c r="D38" s="2" t="inlineStr">
         <is>
-          <t>Akela Hotel Gym</t>
+          <t>if rohit≥44</t>
         </is>
       </c>
       <c r="E38" s="2" t="inlineStr">
         <is>
-          <t>if rohit≥44</t>
-        </is>
-      </c>
-      <c r="F38" s="2" t="inlineStr">
-        <is>
           <t>A</t>
         </is>
       </c>
-      <c r="G38" s="3" t="inlineStr">
+      <c r="F38" s="3" t="inlineStr">
         <is>
           <t>Full surrender — jo bolo, wahi</t>
         </is>
       </c>
-      <c r="H38" s="10" t="n">
+      <c r="G38" s="10" t="n">
         <v>4</v>
       </c>
+      <c r="H38" s="4" t="n">
+        <v>0</v>
+      </c>
       <c r="I38" s="4" t="n">
         <v>0</v>
       </c>
-      <c r="J38" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="K38" s="3" t="inlineStr">
+      <c r="J38" s="3" t="inlineStr">
         <is>
           <t>rohit +3</t>
         </is>
       </c>
-      <c r="L38" s="3" t="inlineStr"/>
+      <c r="K38" s="2" t="inlineStr">
+        <is>
+          <t>DM</t>
+        </is>
+      </c>
+      <c r="L38" s="2" t="inlineStr">
+        <is>
+          <t>rohit</t>
+        </is>
+      </c>
+      <c r="M38" s="3" t="inlineStr">
+        <is>
+          <t>Shot tha. Ball nahi thi. Ab dono milenge. Kal same time.</t>
+        </is>
+      </c>
+      <c r="N38" s="3" t="inlineStr"/>
+      <c r="O38" s="3" t="inlineStr">
+        <is>
+          <t>coach: Slump technique se kam, sochne ke tareeke se zyada tootta hai. Mere har student ko ek hi …</t>
+        </is>
+      </c>
+      <c r="P38" s="3" t="inlineStr"/>
+      <c r="Q38" s="2" t="inlineStr"/>
     </row>
     <row r="39">
       <c r="A39" s="6" t="inlineStr">
@@ -2408,44 +2985,57 @@
       </c>
       <c r="C39" s="6" t="inlineStr">
         <is>
-          <t>The Reckoning</t>
+          <t>Akela Hotel Gym</t>
         </is>
       </c>
       <c r="D39" s="6" t="inlineStr">
         <is>
-          <t>Akela Hotel Gym</t>
+          <t>if rohit≥44</t>
         </is>
       </c>
       <c r="E39" s="6" t="inlineStr">
         <is>
-          <t>if rohit≥44</t>
-        </is>
-      </c>
-      <c r="F39" s="6" t="inlineStr">
-        <is>
           <t>B</t>
         </is>
       </c>
-      <c r="G39" s="7" t="inlineStr">
+      <c r="F39" s="7" t="inlineStr">
         <is>
           <t>Apna tareeka defend karo</t>
         </is>
       </c>
-      <c r="H39" s="9" t="n">
-        <v>2</v>
+      <c r="G39" s="9" t="n">
+        <v>2</v>
+      </c>
+      <c r="H39" s="8" t="n">
+        <v>0</v>
       </c>
       <c r="I39" s="8" t="n">
         <v>0</v>
       </c>
-      <c r="J39" s="8" t="n">
-        <v>0</v>
-      </c>
-      <c r="K39" s="7" t="inlineStr">
+      <c r="J39" s="7" t="inlineStr">
         <is>
           <t>rohit -2</t>
         </is>
       </c>
-      <c r="L39" s="7" t="inlineStr"/>
+      <c r="K39" s="6" t="inlineStr">
+        <is>
+          <t>POST</t>
+        </is>
+      </c>
+      <c r="L39" s="6" t="inlineStr"/>
+      <c r="M39" s="7" t="inlineStr"/>
+      <c r="N39" s="7" t="inlineStr">
+        <is>
+          <t>paltanpulse: LONG LENS, 6:14 AM, Wankhede: Rohit Sharma aur woh 16-saal ka ladka. Khaali stadium. Aur …</t>
+        </is>
+      </c>
+      <c r="O39" s="7" t="inlineStr">
+        <is>
+          <t>friend: Bhai 5 baje gym story daal raha hai. Main 5 baje so raha hoon. We are not the same. (Prou…</t>
+        </is>
+      </c>
+      <c r="P39" s="7" t="inlineStr"/>
+      <c r="Q39" s="6" t="inlineStr"/>
     </row>
     <row r="40">
       <c r="A40" s="2" t="inlineStr">
@@ -2458,44 +3048,61 @@
       </c>
       <c r="C40" s="2" t="inlineStr">
         <is>
-          <t>The Reckoning</t>
+          <t>Do Naam, Ek Jagah</t>
         </is>
       </c>
       <c r="D40" s="2" t="inlineStr">
         <is>
-          <t>Do Naam, Ek Jagah</t>
+          <t>default</t>
         </is>
       </c>
       <c r="E40" s="2" t="inlineStr">
         <is>
-          <t>default</t>
-        </is>
-      </c>
-      <c r="F40" s="2" t="inlineStr">
-        <is>
           <t>A</t>
         </is>
       </c>
-      <c r="G40" s="3" t="inlineStr">
+      <c r="F40" s="3" t="inlineStr">
         <is>
           <t>Naman ke saath prep karo</t>
         </is>
       </c>
-      <c r="H40" s="10" t="n">
+      <c r="G40" s="10" t="n">
         <v>1</v>
       </c>
-      <c r="I40" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="J40" s="10" t="n">
+      <c r="H40" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="I40" s="10" t="n">
         <v>3</v>
       </c>
-      <c r="K40" s="3" t="inlineStr">
+      <c r="J40" s="3" t="inlineStr">
         <is>
           <t>naman +4, tilak +2</t>
         </is>
       </c>
-      <c r="L40" s="3" t="inlineStr"/>
+      <c r="K40" s="2" t="inlineStr">
+        <is>
+          <t>DM</t>
+        </is>
+      </c>
+      <c r="L40" s="2" t="inlineStr">
+        <is>
+          <t>naman ×3</t>
+        </is>
+      </c>
+      <c r="M40" s="3" t="inlineStr">
+        <is>
+          <t>Bro tu aa gaya. Sach bolun? Mujhe laga nahi tha tu aayega. 😅 | Ok sun — maine unke death bowler ka poora season dekha hai. 19th over: pehli 3 gendein…</t>
+        </is>
+      </c>
+      <c r="N40" s="3" t="inlineStr"/>
+      <c r="O40" s="3" t="inlineStr">
+        <is>
+          <t>tilak: 2 naam, 1 jagah — aur dono aaj saath nets pe the. Yeh hota hai dressing room culture. 💙</t>
+        </is>
+      </c>
+      <c r="P40" s="3" t="inlineStr"/>
+      <c r="Q40" s="2" t="inlineStr"/>
     </row>
     <row r="41">
       <c r="A41" s="6" t="inlineStr">
@@ -2508,44 +3115,57 @@
       </c>
       <c r="C41" s="6" t="inlineStr">
         <is>
-          <t>The Reckoning</t>
+          <t>Do Naam, Ek Jagah</t>
         </is>
       </c>
       <c r="D41" s="6" t="inlineStr">
         <is>
-          <t>Do Naam, Ek Jagah</t>
+          <t>default</t>
         </is>
       </c>
       <c r="E41" s="6" t="inlineStr">
         <is>
-          <t>default</t>
-        </is>
-      </c>
-      <c r="F41" s="6" t="inlineStr">
-        <is>
           <t>B</t>
         </is>
       </c>
-      <c r="G41" s="7" t="inlineStr">
+      <c r="F41" s="7" t="inlineStr">
         <is>
           <t>Politics khelo — numbers press ko do</t>
         </is>
       </c>
+      <c r="G41" s="9" t="n">
+        <v>1</v>
+      </c>
       <c r="H41" s="9" t="n">
-        <v>1</v>
-      </c>
-      <c r="I41" s="9" t="n">
         <v>3</v>
       </c>
-      <c r="J41" s="11" t="n">
+      <c r="I41" s="11" t="n">
         <v>-3</v>
       </c>
-      <c r="K41" s="7" t="inlineStr">
+      <c r="J41" s="7" t="inlineStr">
         <is>
           <t>naman -4</t>
         </is>
       </c>
-      <c r="L41" s="7" t="inlineStr"/>
+      <c r="K41" s="6" t="inlineStr">
+        <is>
+          <t>POST</t>
+        </is>
+      </c>
+      <c r="L41" s="6" t="inlineStr"/>
+      <c r="M41" s="7" t="inlineStr"/>
+      <c r="N41" s="7" t="inlineStr">
+        <is>
+          <t>cricketroom_india: SOURCES: MI camp mein Eliminator slot ke liye ek 'numbers war' chal raha hai. Humein ek d… || futurexi: POLL 🗳️ WHO STARTS THE ELIMINATOR? {name} vs Naman Dhir — 1 slot, 2 future stars. 24,318 …</t>
+        </is>
+      </c>
+      <c r="O41" s="7" t="inlineStr">
+        <is>
+          <t>friend: Bro yeh 'sources' kaun hai? 🤔 Mujhe kyu lag raha hai main sources ko personally jaanta ho…</t>
+        </is>
+      </c>
+      <c r="P41" s="7" t="inlineStr"/>
+      <c r="Q41" s="6" t="inlineStr"/>
     </row>
     <row r="42">
       <c r="A42" s="2" t="inlineStr">
@@ -2558,44 +3178,61 @@
       </c>
       <c r="C42" s="2" t="inlineStr">
         <is>
-          <t>The Reckoning</t>
+          <t>Do Naam, Ek Jagah</t>
         </is>
       </c>
       <c r="D42" s="2" t="inlineStr">
         <is>
-          <t>Do Naam, Ek Jagah</t>
+          <t>BENCHED</t>
         </is>
       </c>
       <c r="E42" s="2" t="inlineStr">
         <is>
-          <t>BENCHED path</t>
-        </is>
-      </c>
-      <c r="F42" s="2" t="inlineStr">
-        <is>
           <t>A</t>
         </is>
       </c>
-      <c r="G42" s="3" t="inlineStr">
+      <c r="F42" s="3" t="inlineStr">
         <is>
           <t>Naman ke saath prep — usko kal jitao</t>
         </is>
       </c>
-      <c r="H42" s="10" t="n">
-        <v>2</v>
-      </c>
-      <c r="I42" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="J42" s="10" t="n">
+      <c r="G42" s="10" t="n">
+        <v>2</v>
+      </c>
+      <c r="H42" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="I42" s="10" t="n">
         <v>3</v>
       </c>
-      <c r="K42" s="3" t="inlineStr">
+      <c r="J42" s="3" t="inlineStr">
         <is>
           <t>naman +4, tilak +2</t>
         </is>
       </c>
-      <c r="L42" s="3" t="inlineStr"/>
+      <c r="K42" s="2" t="inlineStr">
+        <is>
+          <t>DM</t>
+        </is>
+      </c>
+      <c r="L42" s="2" t="inlineStr">
+        <is>
+          <t>naman ×3</t>
+        </is>
+      </c>
+      <c r="M42" s="3" t="inlineStr">
+        <is>
+          <t>Bro. Tu bench pe hai aur mere liye throw-downs kara raha hai. Yeh main kabhi nahi bhoolunga. | Le, return gift — unka death bowler: 19th over pehli 3…</t>
+        </is>
+      </c>
+      <c r="N42" s="3" t="inlineStr"/>
+      <c r="O42" s="3" t="inlineStr">
+        <is>
+          <t>tilak: 2 naam, 1 jagah — aur dono aaj saath nets pe the. Yeh hota hai dressing room culture. 💙</t>
+        </is>
+      </c>
+      <c r="P42" s="3" t="inlineStr"/>
+      <c r="Q42" s="2" t="inlineStr"/>
     </row>
     <row r="43">
       <c r="A43" s="6" t="inlineStr">
@@ -2608,44 +3245,57 @@
       </c>
       <c r="C43" s="6" t="inlineStr">
         <is>
-          <t>The Reckoning</t>
+          <t>Do Naam, Ek Jagah</t>
         </is>
       </c>
       <c r="D43" s="6" t="inlineStr">
         <is>
-          <t>Do Naam, Ek Jagah</t>
+          <t>BENCHED</t>
         </is>
       </c>
       <c r="E43" s="6" t="inlineStr">
         <is>
-          <t>BENCHED path</t>
-        </is>
-      </c>
-      <c r="F43" s="6" t="inlineStr">
-        <is>
           <t>B</t>
         </is>
       </c>
-      <c r="G43" s="7" t="inlineStr">
+      <c r="F43" s="7" t="inlineStr">
         <is>
           <t>Politics — bahar se pressure banao</t>
         </is>
       </c>
-      <c r="H43" s="8" t="n">
-        <v>0</v>
-      </c>
-      <c r="I43" s="9" t="n">
+      <c r="G43" s="8" t="n">
+        <v>0</v>
+      </c>
+      <c r="H43" s="9" t="n">
         <v>3</v>
       </c>
-      <c r="J43" s="11" t="n">
+      <c r="I43" s="11" t="n">
         <v>-3</v>
       </c>
-      <c r="K43" s="7" t="inlineStr">
+      <c r="J43" s="7" t="inlineStr">
         <is>
           <t>naman -4, mahela -2</t>
         </is>
       </c>
-      <c r="L43" s="7" t="inlineStr"/>
+      <c r="K43" s="6" t="inlineStr">
+        <is>
+          <t>POST</t>
+        </is>
+      </c>
+      <c r="L43" s="6" t="inlineStr"/>
+      <c r="M43" s="7" t="inlineStr"/>
+      <c r="N43" s="7" t="inlineStr">
+        <is>
+          <t>cricketroom_india: SOURCES: MI ke bench pe baitha young batter {name} 'internal numbers' mein squad ke kai n… || futurexi: POLL 🗳️ SHOULD MI RECALL THE KID FOR THE ELIMINATOR? {name} vs current XI — 19,204 votes.…</t>
+        </is>
+      </c>
+      <c r="O43" s="7" t="inlineStr">
+        <is>
+          <t>friend: Bro yeh 'sources' kaun hai? 🤔 Mujhe kyu lag raha hai main sources ko personally jaanta ho…</t>
+        </is>
+      </c>
+      <c r="P43" s="7" t="inlineStr"/>
+      <c r="Q43" s="6" t="inlineStr"/>
     </row>
     <row r="44">
       <c r="A44" s="2" t="inlineStr">
@@ -2658,46 +3308,59 @@
       </c>
       <c r="C44" s="2" t="inlineStr">
         <is>
-          <t>The Reckoning</t>
+          <t>Aakhri Gend Tak</t>
         </is>
       </c>
       <c r="D44" s="2" t="inlineStr">
         <is>
-          <t>Aakhri Gend Tak</t>
+          <t>default</t>
         </is>
       </c>
       <c r="E44" s="2" t="inlineStr">
         <is>
-          <t>default</t>
-        </is>
-      </c>
-      <c r="F44" s="2" t="inlineStr">
-        <is>
           <t>A</t>
         </is>
       </c>
-      <c r="G44" s="3" t="inlineStr">
+      <c r="F44" s="3" t="inlineStr">
         <is>
           <t>Deep le jao — calculated</t>
         </is>
       </c>
-      <c r="H44" s="10" t="n">
+      <c r="G44" s="10" t="n">
         <v>3</v>
       </c>
-      <c r="I44" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="J44" s="10" t="n">
+      <c r="H44" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="I44" s="10" t="n">
         <v>4</v>
       </c>
-      <c r="K44" s="3" t="inlineStr">
+      <c r="J44" s="3" t="inlineStr">
         <is>
           <t>rohit +2</t>
         </is>
       </c>
-      <c r="L44" s="3" t="inlineStr">
-        <is>
-          <t>GATE form≥58; assists: naman≥50→-4, bumrah≥36→-2</t>
+      <c r="K44" s="2" t="inlineStr">
+        <is>
+          <t>GATE</t>
+        </is>
+      </c>
+      <c r="L44" s="2" t="inlineStr"/>
+      <c r="M44" s="3" t="inlineStr"/>
+      <c r="N44" s="3" t="inlineStr"/>
+      <c r="O44" s="3" t="inlineStr">
+        <is>
+          <t>rohit: Pressure mein soch dikhti hai, score nahi. Aaj Wankhede ne dono dekhe.</t>
+        </is>
+      </c>
+      <c r="P44" s="3" t="inlineStr">
+        <is>
+          <t>GATE form≥58 | assists: naman≥50→-4, bumrah≥36→-2 | PASS: 'ELIMINATOR JEET LIYA' feed post | FAIL: 'Ladai Sahi Thi' DM hardik ×2</t>
+        </is>
+      </c>
+      <c r="Q44" s="2" t="inlineStr">
+        <is>
+          <t>clutch</t>
         </is>
       </c>
     </row>
@@ -2712,46 +3375,59 @@
       </c>
       <c r="C45" s="6" t="inlineStr">
         <is>
-          <t>The Reckoning</t>
+          <t>Aakhri Gend Tak</t>
         </is>
       </c>
       <c r="D45" s="6" t="inlineStr">
         <is>
-          <t>Aakhri Gend Tak</t>
+          <t>default</t>
         </is>
       </c>
       <c r="E45" s="6" t="inlineStr">
         <is>
-          <t>default</t>
-        </is>
-      </c>
-      <c r="F45" s="6" t="inlineStr">
-        <is>
           <t>B</t>
         </is>
       </c>
-      <c r="G45" s="7" t="inlineStr">
+      <c r="F45" s="7" t="inlineStr">
         <is>
           <t>Counter-attack — abhi maaro</t>
         </is>
       </c>
+      <c r="G45" s="9" t="n">
+        <v>2</v>
+      </c>
       <c r="H45" s="9" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="I45" s="9" t="n">
-        <v>3</v>
-      </c>
-      <c r="J45" s="9" t="n">
-        <v>2</v>
-      </c>
-      <c r="K45" s="7" t="inlineStr">
+        <v>2</v>
+      </c>
+      <c r="J45" s="7" t="inlineStr">
         <is>
           <t>surya +3</t>
         </is>
       </c>
-      <c r="L45" s="7" t="inlineStr">
-        <is>
-          <t>GATE form≥58; assists: naman≥50→-4, bumrah≥36→-2</t>
+      <c r="K45" s="6" t="inlineStr">
+        <is>
+          <t>GATE</t>
+        </is>
+      </c>
+      <c r="L45" s="6" t="inlineStr"/>
+      <c r="M45" s="7" t="inlineStr"/>
+      <c r="N45" s="7" t="inlineStr"/>
+      <c r="O45" s="7" t="inlineStr">
+        <is>
+          <t>surya: Wankhede nights &gt;&gt;&gt; everything. Aaj ka match bahut time tak yaad rahega. 😄💙</t>
+        </is>
+      </c>
+      <c r="P45" s="7" t="inlineStr">
+        <is>
+          <t>GATE form≥58 | assists: naman≥50→-4, bumrah≥36→-2 | PASS: 'WANKHEDE PAGAL HO GAYA' feed post | FAIL: 'Ek Shot Zyada' DM hardik ×2</t>
+        </is>
+      </c>
+      <c r="Q45" s="6" t="inlineStr">
+        <is>
+          <t>clutch</t>
         </is>
       </c>
     </row>
@@ -2766,44 +3442,61 @@
       </c>
       <c r="C46" s="2" t="inlineStr">
         <is>
-          <t>The Reckoning</t>
+          <t>Aakhri Gend Tak</t>
         </is>
       </c>
       <c r="D46" s="2" t="inlineStr">
         <is>
-          <t>Aakhri Gend Tak</t>
+          <t>BENCHED</t>
         </is>
       </c>
       <c r="E46" s="2" t="inlineStr">
         <is>
-          <t>BENCHED path</t>
-        </is>
-      </c>
-      <c r="F46" s="2" t="inlineStr">
-        <is>
           <t>A</t>
         </is>
       </c>
-      <c r="G46" s="3" t="inlineStr">
+      <c r="F46" s="3" t="inlineStr">
         <is>
           <t>Plan do — data aur guts</t>
         </is>
       </c>
-      <c r="H46" s="10" t="n">
+      <c r="G46" s="10" t="n">
         <v>1</v>
       </c>
-      <c r="I46" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="J46" s="10" t="n">
+      <c r="H46" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="I46" s="10" t="n">
         <v>4</v>
       </c>
-      <c r="K46" s="3" t="inlineStr">
+      <c r="J46" s="3" t="inlineStr">
         <is>
           <t>mahela +3</t>
         </is>
       </c>
-      <c r="L46" s="3" t="inlineStr"/>
+      <c r="K46" s="2" t="inlineStr">
+        <is>
+          <t>DM</t>
+        </is>
+      </c>
+      <c r="L46" s="2" t="inlineStr">
+        <is>
+          <t>hardik ×3</t>
+        </is>
+      </c>
+      <c r="M46" s="3" t="inlineStr">
+        <is>
+          <t>Scenes!! Jeet gaye. Aur woh 19th over ka field change — deep point andar, third man upar — woh tera call tha. | Tune aaj bench se match jitaya. Main …</t>
+        </is>
+      </c>
+      <c r="N46" s="3" t="inlineStr"/>
+      <c r="O46" s="3" t="inlineStr">
+        <is>
+          <t>rohit: Pressure mein soch dikhti hai, score nahi. Aaj Wankhede ne dono dekhe.</t>
+        </is>
+      </c>
+      <c r="P46" s="3" t="inlineStr"/>
+      <c r="Q46" s="2" t="inlineStr"/>
     </row>
     <row r="47">
       <c r="A47" s="6" t="inlineStr">
@@ -2816,40 +3509,53 @@
       </c>
       <c r="C47" s="6" t="inlineStr">
         <is>
-          <t>The Reckoning</t>
+          <t>Aakhri Gend Tak</t>
         </is>
       </c>
       <c r="D47" s="6" t="inlineStr">
         <is>
-          <t>Aakhri Gend Tak</t>
+          <t>BENCHED</t>
         </is>
       </c>
       <c r="E47" s="6" t="inlineStr">
         <is>
-          <t>BENCHED path</t>
-        </is>
-      </c>
-      <c r="F47" s="6" t="inlineStr">
-        <is>
           <t>B</t>
         </is>
       </c>
-      <c r="G47" s="7" t="inlineStr">
+      <c r="F47" s="7" t="inlineStr">
         <is>
           <t>Camera dekh ke sulk</t>
         </is>
       </c>
-      <c r="H47" s="8" t="n">
-        <v>0</v>
-      </c>
-      <c r="I47" s="9" t="n">
+      <c r="G47" s="8" t="n">
+        <v>0</v>
+      </c>
+      <c r="H47" s="9" t="n">
         <v>1</v>
       </c>
-      <c r="J47" s="11" t="n">
+      <c r="I47" s="11" t="n">
         <v>-4</v>
       </c>
-      <c r="K47" s="7" t="inlineStr"/>
-      <c r="L47" s="7" t="inlineStr"/>
+      <c r="J47" s="7" t="inlineStr"/>
+      <c r="K47" s="6" t="inlineStr">
+        <is>
+          <t>POST</t>
+        </is>
+      </c>
+      <c r="L47" s="6" t="inlineStr"/>
+      <c r="M47" s="7" t="inlineStr"/>
+      <c r="N47" s="7" t="inlineStr">
+        <is>
+          <t>memeovers: BROADCAST ne LIVE Eliminator mein MI ke young kid ka face pakad liya jab captain bench se…</t>
+        </is>
+      </c>
+      <c r="O47" s="7" t="inlineStr">
+        <is>
+          <t>surya: Wankhede nights &gt;&gt;&gt; everything. Aaj ka match bahut time tak yaad rahega. 😄💙</t>
+        </is>
+      </c>
+      <c r="P47" s="7" t="inlineStr"/>
+      <c r="Q47" s="6" t="inlineStr"/>
     </row>
     <row r="48">
       <c r="A48" s="2" t="inlineStr">
@@ -2862,44 +3568,61 @@
       </c>
       <c r="C48" s="2" t="inlineStr">
         <is>
-          <t>The Reckoning</t>
+          <t>The Verdict</t>
         </is>
       </c>
       <c r="D48" s="2" t="inlineStr">
         <is>
-          <t>The Verdict</t>
+          <t>default</t>
         </is>
       </c>
       <c r="E48" s="2" t="inlineStr">
         <is>
-          <t>default</t>
-        </is>
-      </c>
-      <c r="F48" s="2" t="inlineStr">
-        <is>
           <t>A</t>
         </is>
       </c>
-      <c r="G48" s="3" t="inlineStr">
+      <c r="F48" s="3" t="inlineStr">
         <is>
           <t>Phone off — Coach ke academy jao</t>
         </is>
       </c>
+      <c r="G48" s="4" t="n">
+        <v>0</v>
+      </c>
       <c r="H48" s="4" t="n">
         <v>0</v>
       </c>
-      <c r="I48" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="J48" s="10" t="n">
+      <c r="I48" s="10" t="n">
         <v>1</v>
       </c>
-      <c r="K48" s="3" t="inlineStr">
+      <c r="J48" s="3" t="inlineStr">
         <is>
           <t>coach +3</t>
         </is>
       </c>
-      <c r="L48" s="3" t="inlineStr"/>
+      <c r="K48" s="2" t="inlineStr">
+        <is>
+          <t>DM</t>
+        </is>
+      </c>
+      <c r="L48" s="2" t="inlineStr">
+        <is>
+          <t>coach ×3</t>
+        </is>
+      </c>
+      <c r="M48" s="3" t="inlineStr">
+        <is>
+          <t>Aa gaya? Pad pehen. Phone mere pocket mein rahega — 6 baje tak sirf throwdowns. Jaise gyaarah saal ki umar mein. | Yaad hai pehli season ball? Ro rah…</t>
+        </is>
+      </c>
+      <c r="N48" s="3" t="inlineStr"/>
+      <c r="O48" s="3" t="inlineStr">
+        <is>
+          <t>friend: Bro ne verdict day pe phone OFF karke academy chala gaya. Main uski jagah stress le raha …</t>
+        </is>
+      </c>
+      <c r="P48" s="3" t="inlineStr"/>
+      <c r="Q48" s="2" t="inlineStr"/>
     </row>
     <row r="49">
       <c r="A49" s="6" t="inlineStr">
@@ -2912,43 +3635,56 @@
       </c>
       <c r="C49" s="6" t="inlineStr">
         <is>
-          <t>The Reckoning</t>
+          <t>The Verdict</t>
         </is>
       </c>
       <c r="D49" s="6" t="inlineStr">
         <is>
-          <t>The Verdict</t>
+          <t>default</t>
         </is>
       </c>
       <c r="E49" s="6" t="inlineStr">
         <is>
-          <t>default</t>
-        </is>
-      </c>
-      <c r="F49" s="6" t="inlineStr">
-        <is>
           <t>B</t>
         </is>
       </c>
-      <c r="G49" s="7" t="inlineStr">
+      <c r="F49" s="7" t="inlineStr">
         <is>
           <t>Live tracker + statement ready</t>
         </is>
       </c>
-      <c r="H49" s="8" t="n">
-        <v>0</v>
-      </c>
-      <c r="I49" s="9" t="n">
-        <v>2</v>
-      </c>
-      <c r="J49" s="11" t="n">
+      <c r="G49" s="8" t="n">
+        <v>0</v>
+      </c>
+      <c r="H49" s="9" t="n">
+        <v>2</v>
+      </c>
+      <c r="I49" s="11" t="n">
         <v>-1</v>
       </c>
-      <c r="K49" s="7" t="inlineStr"/>
-      <c r="L49" s="7" t="inlineStr"/>
+      <c r="J49" s="7" t="inlineStr"/>
+      <c r="K49" s="6" t="inlineStr">
+        <is>
+          <t>POST</t>
+        </is>
+      </c>
+      <c r="L49" s="6" t="inlineStr"/>
+      <c r="M49" s="7" t="inlineStr"/>
+      <c r="N49" s="7" t="inlineStr">
+        <is>
+          <t>YOU: Jo bhi 6 baje ho — yeh season maine kamaaya hai, maanga nahi. Mumbai ne mujhe khareeda th…</t>
+        </is>
+      </c>
+      <c r="O49" s="7" t="inlineStr">
+        <is>
+          <t>coach: Aaj ke din bhi post pehle aayi, call baad mein. Zamana badal gaya. Number wahi hai beta —…</t>
+        </is>
+      </c>
+      <c r="P49" s="7" t="inlineStr"/>
+      <c r="Q49" s="6" t="inlineStr"/>
     </row>
   </sheetData>
-  <autoFilter ref="A1:L1"/>
+  <autoFilter ref="A1:Q1"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -2959,19 +3695,19 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D24"/>
+  <dimension ref="A1:D21"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="42" customWidth="1" min="1" max="1"/>
-    <col width="40" customWidth="1" min="2" max="2"/>
-    <col width="24" customWidth="1" min="3" max="3"/>
-    <col width="22" customWidth="1" min="4" max="4"/>
+    <col width="46" customWidth="1" min="1" max="1"/>
+    <col width="60" customWidth="1" min="2" max="2"/>
+    <col width="22" customWidth="1" min="3" max="3"/>
+    <col width="20" customWidth="1" min="4" max="4"/>
   </cols>
   <sheetData>
     <row r="1">
       <c r="A1" s="12" t="inlineStr">
         <is>
-          <t>LORE — Indian Dressing Room · metric reference</t>
+          <t>LORE — Indian Dressing Room · reference</t>
         </is>
       </c>
       <c r="B1" t="inlineStr"/>
@@ -2981,7 +3717,7 @@
       <c r="B2" t="inlineStr"/>
     </row>
     <row r="3">
-      <c r="A3" s="13" t="inlineStr">
+      <c r="A3" t="inlineStr">
         <is>
           <t>STARTING VALUES</t>
         </is>
@@ -2991,7 +3727,7 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>Form (goal 1)</t>
+          <t>Form</t>
         </is>
       </c>
       <c r="B4" t="n">
@@ -3001,7 +3737,7 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>Captain's Trust = dmTrust.hardik (goal 2)</t>
+          <t>Captain's Trust (dmTrust.hardik)</t>
         </is>
       </c>
       <c r="B5" t="n">
@@ -3011,7 +3747,7 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>Fame / followers (secondary)</t>
+          <t>Fame</t>
         </is>
       </c>
       <c r="B6" t="n">
@@ -3023,9 +3759,9 @@
       <c r="B7" t="inlineStr"/>
     </row>
     <row r="8">
-      <c r="A8" s="13" t="inlineStr">
-        <is>
-          <t>HOW METRICS MOVE</t>
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>ONE OUTCOME PER CHOICE</t>
         </is>
       </c>
       <c r="B8" t="inlineStr"/>
@@ -3033,208 +3769,172 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>Form</t>
+          <t>Each choice fires EITHER a DM (to a character) OR a Post (yours/authored) — never both.</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>ONLY via choice deltas.form (matches, nets, decisions)</t>
+          <t>The beat's feedReaction always adds a reaction post on top. Gated beats (S7,S13) branch pass/fail, each with its own DM/post.</t>
         </is>
       </c>
     </row>
     <row r="10">
-      <c r="A10" t="inlineStr">
-        <is>
-          <t>Captain's Trust</t>
-        </is>
-      </c>
-      <c r="B10" t="inlineStr">
-        <is>
-          <t>choice relationshipDeltas.hardik + DM chat with Hardik (cap +4/window) + trust moments</t>
-        </is>
-      </c>
+      <c r="A10" t="inlineStr"/>
+      <c r="B10" t="inlineStr"/>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>Fame</t>
-        </is>
-      </c>
-      <c r="B11" t="inlineStr">
-        <is>
-          <t>choice deltas.fame + posting captions + comment replies</t>
-        </is>
-      </c>
+          <t>SELECTION THRESHOLDS</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr"/>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>Other seniors</t>
+          <t>Week</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>their own relationshipDeltas — unlock advice, assists, warmth</t>
+          <t>START</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>LIFELINE</t>
+        </is>
+      </c>
+      <c r="D12" t="inlineStr">
+        <is>
+          <t>Recall</t>
         </is>
       </c>
     </row>
     <row r="13">
-      <c r="A13" t="inlineStr"/>
-      <c r="B13" t="inlineStr"/>
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>W1</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>form≥44 &amp; captain≥34</t>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>form≥38 &amp; captain≥40</t>
+        </is>
+      </c>
+      <c r="D13" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
     </row>
     <row r="14">
-      <c r="A14" s="13" t="inlineStr">
-        <is>
-          <t>SELECTION THRESHOLDS (squad verdict at each week end)</t>
-        </is>
-      </c>
-      <c r="B14" t="inlineStr"/>
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>W2</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>form≥52 &amp; captain≥44</t>
+        </is>
+      </c>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>form≥46 &amp; captain≥52</t>
+        </is>
+      </c>
+      <c r="D14" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
     </row>
     <row r="15">
-      <c r="A15" s="14" t="inlineStr">
-        <is>
-          <t>Week</t>
-        </is>
-      </c>
-      <c r="B15" s="14" t="inlineStr">
-        <is>
-          <t>START needs</t>
-        </is>
-      </c>
-      <c r="C15" s="14" t="inlineStr">
-        <is>
-          <t>LIFELINE needs</t>
-        </is>
-      </c>
-      <c r="D15" s="14" t="inlineStr">
-        <is>
-          <t>Recall</t>
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>W3</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>form≥58 &amp; captain≥52</t>
+        </is>
+      </c>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>form≥48 &amp; captain≥58</t>
+        </is>
+      </c>
+      <c r="D15" t="inlineStr">
+        <is>
+          <t>benched→ form≥56</t>
         </is>
       </c>
     </row>
     <row r="16">
-      <c r="A16" t="inlineStr">
-        <is>
-          <t>W1 (after S4)</t>
-        </is>
-      </c>
-      <c r="B16" t="inlineStr">
-        <is>
-          <t>form≥44 &amp; captain≥34</t>
-        </is>
-      </c>
-      <c r="C16" t="inlineStr">
-        <is>
-          <t>form≥38 &amp; captain≥40</t>
-        </is>
-      </c>
-      <c r="D16" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
+      <c r="A16" t="inlineStr"/>
+      <c r="B16" t="inlineStr"/>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>W2 (after S9)</t>
-        </is>
-      </c>
-      <c r="B17" t="inlineStr">
-        <is>
-          <t>form≥52 &amp; captain≥44</t>
-        </is>
-      </c>
-      <c r="C17" t="inlineStr">
-        <is>
-          <t>form≥46 &amp; captain≥52</t>
-        </is>
-      </c>
-      <c r="D17" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
+          <t>ENDINGS</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr"/>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>W3 (after S12)</t>
+          <t>The Call-Up</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>form≥58 &amp; captain≥52</t>
-        </is>
-      </c>
-      <c r="C18" t="inlineStr">
-        <is>
-          <t>form≥48 &amp; captain≥58</t>
-        </is>
-      </c>
-      <c r="D18" t="inlineStr">
-        <is>
-          <t>benched→ form≥56</t>
+          <t>form≥58 &amp; captain≥55 &amp; benched≤1</t>
         </is>
       </c>
     </row>
     <row r="19">
-      <c r="A19" t="inlineStr"/>
-      <c r="B19" t="inlineStr"/>
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>Captain's Bet</t>
+        </is>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>captain≥55 &amp; (form≥48 or captain≥60)</t>
+        </is>
+      </c>
     </row>
     <row r="20">
-      <c r="A20" s="13" t="inlineStr">
-        <is>
-          <t>ENDINGS (from final form / captain / times benched)</t>
-        </is>
-      </c>
-      <c r="B20" t="inlineStr"/>
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>Stats Machine</t>
+        </is>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>form≥58 (captain &lt;55)</t>
+        </is>
+      </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>The Call-Up</t>
+          <t>Not Yet</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>form≥58 &amp; captain≥55 &amp; benched≤1</t>
-        </is>
-      </c>
-    </row>
-    <row r="22">
-      <c r="A22" t="inlineStr">
-        <is>
-          <t>Captain's Bet</t>
-        </is>
-      </c>
-      <c r="B22" t="inlineStr">
-        <is>
-          <t>captain≥55 &amp; (form≥48 or captain≥60)</t>
-        </is>
-      </c>
-    </row>
-    <row r="23">
-      <c r="A23" t="inlineStr">
-        <is>
-          <t>Stats Machine</t>
-        </is>
-      </c>
-      <c r="B23" t="inlineStr">
-        <is>
-          <t>form≥58 (captain &lt;55)</t>
-        </is>
-      </c>
-    </row>
-    <row r="24">
-      <c r="A24" t="inlineStr">
-        <is>
-          <t>Not Yet</t>
-        </is>
-      </c>
-      <c r="B24" t="inlineStr">
-        <is>
-          <t>else; forced if benched twice &amp; captain &lt;60</t>
+          <t>else; forced if benched×2 &amp; captain&lt;60</t>
         </is>
       </c>
     </row>

</xml_diff>